<commit_message>
feat: add exam strategy guide and update study checklist for CCA-F preparation
</commit_message>
<xml_diff>
--- a/CCAF-Study-Checklist.xlsx
+++ b/CCAF-Study-Checklist.xlsx
@@ -1,23 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\Russel-QL2\_Dev\Claude-Learning-Exercises\CCAF-StudyGuide\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DEDC5DE-1A39-4B71-ACD4-6018B70C8340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Checklist" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Objective Map" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Checklist" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
+    <sheet name="Objective Map" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Checklist!$A$1:$K$61</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Objective Map'!$A$4:$E$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Checklist!$A$1:$K$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Objective Map'!$A$4:$E$41</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -28,841 +44,839 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="275">
   <si>
-    <t xml:space="preserve">Phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Domain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resource (click to open)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Est (h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P0 - Orient</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HIGH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read the kit README, then skim the official links index so you know where everything lives</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Setup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01 - Official links index</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not Started</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Download the official Exam Guide PDF; do all 12 sample questions reading every wrong-answer rationale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skilljar - CCA-F certification page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60 questions / 120 min / passing score 720. Domain weights: D1 27, D3 20, D4 20, D2 18, D5 15 (%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read the exam-day one-pager once now (you will reread it in the final 24h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strategy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05 - Exam-day one-pager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The enforcement ladder and wrong-answer tells frame everything that follows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1 - D1 Agentic Architecture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline drill: D1 filter, 5 questions; note which misses were honeypots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02 - Honeypot drill (open in browser)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read: Building effective agents - workflows vs agents; the five workflow patterns incl. orchestrator-workers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anthropic engineering post</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covers the tested objectives on orchestration pattern selection and when-to-build-an-agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read: How we built our multi-agent research system</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covers subagent prompt completeness, checkpoints / state persistence, resume-on-error, orchestrator-worker in production - all tested objectives</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Tool use overview - the agent loop, stop_reason values, parallel tool use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs - Tool use overview</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loop control: stop_reason drives everything; NL-parsing and iteration caps are wrong-answer tells</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Subagents in Claude Code - context isolation, tool restrictions, spawning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Subagents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subagents inherit nothing from the parent; spawn prompts must be complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 10: Orchestrator-worker isolation &amp; provenance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03 - Labs index (domain-labs.md)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 11: The agent loop done right</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 12: Agent design judgment - tiering, error contracts, escalation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-drill D1 the next day; must hold 5/5, else revisit rationales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2 - D2 Tool Design &amp; MCP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline drill: D2 filter, 5 questions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Tool use overview - descriptions / when-to-call, tool_choice modes, strict</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same page as the D1 pass; this pass focuses on tool descriptions, tool_choice and strict</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: MCP in Claude Code - scopes (local/project/user), env-var expansion, /mcp, auth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - MCP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Also know MCP resources vs tools (tested); concepts at modelcontextprotocol.io</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Courses: Intro to MCP + MCP Advanced Topics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Course</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Academy - Intro to MCP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 13: Tool definitions that trigger correctly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 14: Scoped tools &amp; parallel execution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 15: MCP integration (needs Node / npx)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-drill D2; must hold 5/5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P3 - D3 Claude Code Config</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline drill: D3 filter, 5 questions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Extend Claude Code - when to use CLAUDE.md vs rules vs skills vs subagents vs hooks vs MCP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Extend Claude Code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Directly covers the tested config-mechanism-selection objective</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Memory - CLAUDE.md hierarchy (managed/user/project), subdirectory loading, @imports, .claude/rules/ with paths globs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Memory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tip: set CLAUDE_CODE_NEW_INIT=1 for the interactive multi-phase /init flow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Hooks - events, matchers, exit codes (PreToolUse exit 2 blocks)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Hooks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Skills - SKILL.md frontmatter, progressive disclosure, triggering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Skills</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tip: study the skill-creator skill as a worked example of good frontmatter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Slash commands vs skills - when you invoke vs when Claude does</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Slash commands</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Settings and permissions - allow/deny rules, settings scopes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Settings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tip: the $schema line in settings.json enables autocomplete + inline validation in editors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Permission modes incl. plan mode - plan vs direct execution vs multi-phase review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Permission modes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covers the tested review-architecture objective: choose by task scope, risk level, approval requirements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: CLI reference + Headless - -p, --output-format json, --resume, --bare, --tools vs --allowedTools</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - CLI reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Field-note exam question: slow scripted startup -&gt; --bare + --allowedTools (see exam-strategy one-pager); headless page: code.claude.com/docs/en/headless</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Tools reference + Common workflows - Grep vs Glob vs Read vs Bash; incremental codebase exploration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Tools reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covers the tested built-in-tool-selection + exploration-strategy objectives; workflows: code.claude.com/docs/en/common-workflows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Sessions (--continue/--resume scope rules) + Code review configuration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - Sessions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review configs (standards, tool restriction, structured output) are a tested objective; see code.claude.com/docs/en/code-review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 4: Memory hierarchy walk + skill triggering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 5: Enforcement, not exhortation (highest-yield lab in the kit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 6: Headless CI with generator/reviewer isolation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Courses: Claude Code in Action; Intro to Agent Skills; Intro to Subagents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Academy - course catalog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: GitHub Actions integration (CI scenario)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code docs - GitHub Actions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-drill D3; must hold 5/5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P4 - D4 Prompt Eng &amp; Output</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline drill: D4 filter, 5 questions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Study Prompting best practices end to end (examples, chaining, agentic prompting)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs - Prompting best practices</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Study Structured outputs; memorize: citations+format=400, prefill incompatible, format change kills cache, strict+JSON combinable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs - Structured outputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Also covers extraction-schema design with optional/nullable fields and enums (tested objective)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 1: Break JSON on purpose, then make it unbreakable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 2: Strict tool use and schema drift</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 3: Validation-retry loop and example diversity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hands-on with Console prompting tools: generator, improver, evaluation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs - Console prompting tools</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Course: Building with the Claude API (find in Academy catalog)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-drill D4; must hold 5/5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P5 - D5 Context &amp; Reliability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline drill: D5 filter, 5 questions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Context editing - tool-result clearing, thinking clearing, compaction summary structure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs - Context editing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extra reading: joeyyu23.github.io/claude-code-handbook (architect / harness engineering)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read: Effective context engineering for AI agents (engineering post)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 7: Prompt caching forensics (prefix invalidation signatures)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 8: Context editing under tool-call load</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 9: stop_reason handling + compaction contract</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs: Batch processing - sync vs batch decision, custom_id, 24h window</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docs - Batch processing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-drill D5; must hold 5/5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6 - Final Prep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review 12-week repo: Key Anti-Patterns and Decision Frameworks tables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Community</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GitHub - SGridworks 12-week program</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unofficial; when it disagrees with the docs, the docs win</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full 25-question honeypot drill, shuffled, cold; target 21+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Community mock: 60-question simulator (unofficial; pattern practice only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Practice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anthropiccertifications.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12-week repo practice tests (110 questions in practice-tests/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GitHub - repo practice-tests folder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Official Skilljar practice exam, final pass; read EVERY rationale incl. correct answers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day before: exam-strategy one-pager + terminology hit list; no new material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCA-F Prep Dashboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overall progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hours remaining</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Progress by phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Progress by domain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exam weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D1 - Agentic Architecture &amp; Orchestration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D2 - Tool Design &amp; MCP Integration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3 - Claude Code Config &amp; Workflows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D4 - Prompt Eng &amp; Structured Output</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D5 - Context Mgmt &amp; Reliability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cross-domain (orient + final prep)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How to use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Work the Checklist tab top to bottom: P0 orientation, then one domain phase at a time (D1 through D5, ordered by domain number), then P6 final prep.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Edit ONLY the three input columns: Status (dropdown), Date done, and Notes. Every other cell, and this dashboard, is formula-driven.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Example entry: when you finish a task, set Status = Done and Date done = 2026-07-15 (any date format works); the row tints green and the Dashboard updates.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Status colors: green = Done, amber = In Progress. Red priority text = HIGH.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Resource links open docs and courses online; drill, labs, and strategy links open local files in this kit (keep the workbook in the kit's root folder).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Lab answer keys live in 03-Hands-On-Labs/_AnswerKeys/ - attempt each lab before opening its key.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exam objective coverage map</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test objectives from the official exam blueprint (as reported section-wise on score reports). Each objective is mapped to where this kit covers it; doc coverage verified against the linked pages (July 2026).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exam objective</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covered in this kit by</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primary reference (click to open)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configure agentic loops to emit multiple tool calls within a single response turn, enabling parallel execution of independent subtasks and reducing total round-trip latency.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 11 step 4 - Lab 14 step 3 - Drill Q16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool use overview</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply session resumption techniques - including targeted re-analysis of changed files and context injection - to restore agent state accurately without repeating prior work.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checklist P3 Sessions row - Strategy sheet 'State persistence'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sessions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Construct subagent prompts that include all findings, structured data, and source metadata required for task completion without returning to the coordinator for missing context.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 10 steps 1-2 - Drill Q17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How we built our multi-agent research system</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluate subagent delegation strategies - goal-oriented versus procedural instructions - and select the approach that enables adaptive behavior while maintaining coordinator visibility and control.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strategy sheet 'Multi-agent' (delegation style)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multi-agent research post ('Teach the orchestrator how to delegate')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configure subagent invocations with appropriate tool restrictions, context scoping, and system prompts that constrain each agent to its designated role.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 10 - Lab 14 - Drill Q23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subagents in Claude Code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diagnose misconfigured subagent spawning by identifying missing tool permissions, incorrect AgentDefinition parameters, or absent coordinator-to-subagent wiring.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Official links index (D1 section)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subagents in the Agent SDK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decompose complex tasks into dynamically generated subtasks that adapt as new information is discovered, rather than executing a fixed sequence regardless of intermediate findings.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drill Q18 - Lab 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Building effective agents (orchestrator-workers)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select the appropriate agentic review architecture - plan mode, direct execution, or multi-phase workflow - based on task scope, risk level, and human approval requirements.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checklist P3 Permission-modes row - Strategy sheet 'Review architecture'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permission modes (incl. plan mode)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design state persistence strategies for multi-agent pipelines that enable reliable resumption after interruption without repeating completed work or losing prior findings.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drill Q19 - Strategy sheet 'State persistence'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multi-agent research post (checkpoints, resume-on-error)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluate multi-agent orchestration patterns - coordinator-worker, parallel execution, and sequential pipelines - to select the structure best satisfying research coverage, latency, and reliability requirements.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Building effective agents (the five workflow patterns)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configure Claude Code CLI invocations for automated CI/CD pipelines using non-interactive flags, permission modes, and cost and turn limits that prevent runaway executions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 6 - Drill Q9 - Strategy sheet field note (--bare)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLI reference + Headless</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Structure iterative refinement workflows by providing concrete input-output examples, targeted feedback on specific failures, and batched issue descriptions for consolidated evaluation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 3 (validation-retry, targeted feedback)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prompting best practices</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design Claude Code review configurations that load the correct project standards, restrict unnecessary tool access, and produce structured output suitable for automated downstream processing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 6 (two-stage pipeline) - Checklist P3 Sessions/Code-review row</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply the context: fork frontmatter option to Skill and slash command configurations that should execute in an isolated subagent context, preventing cross-contamination of session state.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strategy sheet 'Slash command vs skill vs subagent' - Checklist P3 Skills row</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skills ('Run skills in a subagent')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Improve automated test generation quality by providing existing test files as context, defining fixture conventions, and specifying criteria that distinguish meaningful behavioral tests from trivial assertions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checklist P3 Tools-reference/Common-workflows row</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Common workflows (testing)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select the correct Claude Code configuration mechanism - CLAUDE.md, .claude/rules/ with glob patterns, Skills, hooks, or settings permissions - based on guidance type and when it should apply.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labs 4-5 - Drill Q6-Q8, Q10 - Strategy sheet 'Config mechanism selection'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extend Claude Code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply systematic codebase exploration strategies using Grep, Glob, and Read tools that build incremental understanding while managing context window constraints.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strategy sheet 'Built-in tool selection'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Common workflows + Tools reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design subagent output schemas that render structured data, prose summaries, and citation metadata in the format best suited to downstream synthesis and reporting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 10 (Finding schema)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multi-agent research post (appendix: subagent outputs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design synthesis agent behavior that preserves source-level uncertainty, distinguishing well-established findings from contested claims rather than collapsing conflicting data into single confident statements.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 10 step 4 (provenance) - Drill Q14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multi-agent research post</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply context management strategies - subagent isolation, scratchpad files, and targeted file reading - to sustain coherent codebase exploration across sessions exceeding context limits.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 8 - Lab 10 (isolation)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Effective context engineering for AI agents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply context window optimization techniques - summarization, sliding windows, structured state objects, and selective retention - to maintain response quality as conversations exceed practical token limits.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labs 8-9 - Drill Q11, Q15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Context editing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design human review routing strategies that direct extractions to reviewers based on confidence scores, document characteristics, and field-level ambiguity rather than random sampling.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strategy sheet 'Human review routing' - Lab 12 part 3 (signal quality)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exam-day one-pager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select the appropriate API processing mode - synchronous Messages API or asynchronous Message Batches API - based on latency requirements, workflow blocking behavior, and acceptable processing windows.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checklist P5 Batch row - Strategy sheet 'Headless / CI'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Batch processing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design specialized review passes that separate concerns - security, business logic, API design - into focused prompts with dedicated few-shot examples, preventing recall trade-offs from competing concerns in a single prompt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strategy sheet 'Review architecture' - Drill Q5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select and implement the most reliable structured output method - tool use with JSON schema, prompt-based formatting, or prefilled responses - based on required schema compliance strictness.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 1 - Drill Q1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Structured outputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design extraction schemas with optional fields, nullable values, and appropriate enum definitions that allow the model to accurately represent missing or ambiguous information without fabricating values.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 2 - Checklist P4 Structured-outputs row</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implement tool use with defined JSON schemas to enforce structured output compliance, and configure tool_choice to guarantee tool invocation when conversational responses would cause downstream failures.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 13 - Drill Q22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resolve structured output truncation failures by splitting large review tasks into smaller scoped API calls and merging resulting data structures, rather than increasing max_tokens beyond practical limits.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 9 - Drill Q13 - Strategy sheet 'stop_reason' (split-and-merge)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply extraction accuracy patterns - structured schemas with optional fields, format normalization instructions, and few-shot examples - to reduce hallucination and improve consistency across varied document formats.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labs 1-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Structured outputs + Prompting best practices</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reduce automated review false positive rates by supplying project-specific conventions, accepted patterns, and exclusion criteria as persistent context applied on every review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 4 (CLAUDE.md) - Checklist P3 Memory row</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memory + Code review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design prompt criteria that define explicit inclusion and exclusion boundaries, preventing the model from generating findings or extractions in categories where performance is unreliable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select the appropriate Claude Code built-in tool - Grep, Glob, Read, or Bash - based on the nature of the search or file operation required for a given codebase task.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tools reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configure tool distribution in multi-agent systems by assigning each subagent only the tools required for its designated role, reducing decision complexity and preventing out-of-role tool invocations.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 14 - Drill Q23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subagents + Tool use overview</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distinguish between MCP resources and tools, and expose server content as resources to reduce exploratory tool calls and improve agent efficiency in cross-system queries.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drill Q24 - Lab 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model Context Protocol docs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integrate MCP servers into Claude Code and agent applications by selecting the correct server scope, configuring authentication via environment variable expansion, and verifying tool discovery.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 15 - Drill Q25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCP in Claude Code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write MCP tool descriptions that clearly distinguish each tool's purpose, input formats, use-case boundaries, and relationships to semantically similar tools, reducing misrouting and incorrect tool selection.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 13 - Drill Q21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool use overview + MCP docs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configure the tool_choice parameter to guarantee tool invocation when structured output is required, and sequence multi-tool workflows so prerequisite data is obtained before dependent tools are called.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab 13 step 2 - Drill Q22</t>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Resource (click to open)</t>
+  </si>
+  <si>
+    <t>Est (h)</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Date done</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>P0 - Orient</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>Read the kit README, then skim the official links index so you know where everything lives</t>
+  </si>
+  <si>
+    <t>Setup</t>
+  </si>
+  <si>
+    <t>01 - Official links index</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Download the official Exam Guide PDF; do all 12 sample questions reading every wrong-answer rationale</t>
+  </si>
+  <si>
+    <t>Docs</t>
+  </si>
+  <si>
+    <t>Skilljar - CCA-F certification page</t>
+  </si>
+  <si>
+    <t>60 questions / 120 min / passing score 720. Domain weights: D1 27, D3 20, D4 20, D2 18, D5 15 (%)</t>
+  </si>
+  <si>
+    <t>MED</t>
+  </si>
+  <si>
+    <t>Read the exam-day one-pager once now (you will reread it in the final 24h)</t>
+  </si>
+  <si>
+    <t>Strategy</t>
+  </si>
+  <si>
+    <t>05 - Exam-day one-pager</t>
+  </si>
+  <si>
+    <t>The enforcement ladder and wrong-answer tells frame everything that follows</t>
+  </si>
+  <si>
+    <t>P1 - D1 Agentic Architecture</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>Baseline drill: D1 filter, 5 questions; note which misses were honeypots</t>
+  </si>
+  <si>
+    <t>Drill</t>
+  </si>
+  <si>
+    <t>02 - Honeypot drill (open in browser)</t>
+  </si>
+  <si>
+    <t>Read: Building effective agents - workflows vs agents; the five workflow patterns incl. orchestrator-workers</t>
+  </si>
+  <si>
+    <t>Article</t>
+  </si>
+  <si>
+    <t>Anthropic engineering post</t>
+  </si>
+  <si>
+    <t>Covers the tested objectives on orchestration pattern selection and when-to-build-an-agent</t>
+  </si>
+  <si>
+    <t>Read: How we built our multi-agent research system</t>
+  </si>
+  <si>
+    <t>Covers subagent prompt completeness, checkpoints / state persistence, resume-on-error, orchestrator-worker in production - all tested objectives</t>
+  </si>
+  <si>
+    <t>Docs: Tool use overview - the agent loop, stop_reason values, parallel tool use</t>
+  </si>
+  <si>
+    <t>Docs - Tool use overview</t>
+  </si>
+  <si>
+    <t>Loop control: stop_reason drives everything; NL-parsing and iteration caps are wrong-answer tells</t>
+  </si>
+  <si>
+    <t>Docs: Subagents in Claude Code - context isolation, tool restrictions, spawning</t>
+  </si>
+  <si>
+    <t>Code docs - Subagents</t>
+  </si>
+  <si>
+    <t>Subagents inherit nothing from the parent; spawn prompts must be complete</t>
+  </si>
+  <si>
+    <t>Lab 10: Orchestrator-worker isolation &amp; provenance</t>
+  </si>
+  <si>
+    <t>Lab</t>
+  </si>
+  <si>
+    <t>03 - Labs index (domain-labs.md)</t>
+  </si>
+  <si>
+    <t>Lab 11: The agent loop done right</t>
+  </si>
+  <si>
+    <t>Lab 12: Agent design judgment - tiering, error contracts, escalation</t>
+  </si>
+  <si>
+    <t>Re-drill D1 the next day; must hold 5/5, else revisit rationales</t>
+  </si>
+  <si>
+    <t>P2 - D2 Tool Design &amp; MCP</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>Baseline drill: D2 filter, 5 questions</t>
+  </si>
+  <si>
+    <t>Docs: Tool use overview - descriptions / when-to-call, tool_choice modes, strict</t>
+  </si>
+  <si>
+    <t>Same page as the D1 pass; this pass focuses on tool descriptions, tool_choice and strict</t>
+  </si>
+  <si>
+    <t>Docs: MCP in Claude Code - scopes (local/project/user), env-var expansion, /mcp, auth</t>
+  </si>
+  <si>
+    <t>Code docs - MCP</t>
+  </si>
+  <si>
+    <t>Also know MCP resources vs tools (tested); concepts at modelcontextprotocol.io</t>
+  </si>
+  <si>
+    <t>Courses: Intro to MCP + MCP Advanced Topics</t>
+  </si>
+  <si>
+    <t>Course</t>
+  </si>
+  <si>
+    <t>Academy - Intro to MCP</t>
+  </si>
+  <si>
+    <t>Lab 13: Tool definitions that trigger correctly</t>
+  </si>
+  <si>
+    <t>Lab 14: Scoped tools &amp; parallel execution</t>
+  </si>
+  <si>
+    <t>Lab 15: MCP integration (needs Node / npx)</t>
+  </si>
+  <si>
+    <t>Re-drill D2; must hold 5/5</t>
+  </si>
+  <si>
+    <t>P3 - D3 Claude Code Config</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>Baseline drill: D3 filter, 5 questions</t>
+  </si>
+  <si>
+    <t>Docs: Extend Claude Code - when to use CLAUDE.md vs rules vs skills vs subagents vs hooks vs MCP</t>
+  </si>
+  <si>
+    <t>Code docs - Extend Claude Code</t>
+  </si>
+  <si>
+    <t>Directly covers the tested config-mechanism-selection objective</t>
+  </si>
+  <si>
+    <t>Docs: Memory - CLAUDE.md hierarchy (managed/user/project), subdirectory loading, @imports, .claude/rules/ with paths globs</t>
+  </si>
+  <si>
+    <t>Code docs - Memory</t>
+  </si>
+  <si>
+    <t>Tip: set CLAUDE_CODE_NEW_INIT=1 for the interactive multi-phase /init flow</t>
+  </si>
+  <si>
+    <t>Docs: Hooks - events, matchers, exit codes (PreToolUse exit 2 blocks)</t>
+  </si>
+  <si>
+    <t>Code docs - Hooks</t>
+  </si>
+  <si>
+    <t>Docs: Skills - SKILL.md frontmatter, progressive disclosure, triggering</t>
+  </si>
+  <si>
+    <t>Code docs - Skills</t>
+  </si>
+  <si>
+    <t>Tip: study the skill-creator skill as a worked example of good frontmatter</t>
+  </si>
+  <si>
+    <t>Docs: Slash commands vs skills - when you invoke vs when Claude does</t>
+  </si>
+  <si>
+    <t>Code docs - Slash commands</t>
+  </si>
+  <si>
+    <t>Docs: Settings and permissions - allow/deny rules, settings scopes</t>
+  </si>
+  <si>
+    <t>Code docs - Settings</t>
+  </si>
+  <si>
+    <t>Tip: the $schema line in settings.json enables autocomplete + inline validation in editors</t>
+  </si>
+  <si>
+    <t>Docs: Permission modes incl. plan mode - plan vs direct execution vs multi-phase review</t>
+  </si>
+  <si>
+    <t>Code docs - Permission modes</t>
+  </si>
+  <si>
+    <t>Covers the tested review-architecture objective: choose by task scope, risk level, approval requirements</t>
+  </si>
+  <si>
+    <t>Docs: CLI reference + Headless - -p, --output-format json, --resume, --bare, --tools vs --allowedTools</t>
+  </si>
+  <si>
+    <t>Code docs - CLI reference</t>
+  </si>
+  <si>
+    <t>Field-note exam question: slow scripted startup -&gt; --bare + --allowedTools (see exam-strategy one-pager); headless page: code.claude.com/docs/en/headless</t>
+  </si>
+  <si>
+    <t>Docs: Tools reference + Common workflows - Grep vs Glob vs Read vs Bash; incremental codebase exploration</t>
+  </si>
+  <si>
+    <t>Code docs - Tools reference</t>
+  </si>
+  <si>
+    <t>Covers the tested built-in-tool-selection + exploration-strategy objectives; workflows: code.claude.com/docs/en/common-workflows</t>
+  </si>
+  <si>
+    <t>Docs: Sessions (--continue/--resume scope rules) + Code review configuration</t>
+  </si>
+  <si>
+    <t>Code docs - Sessions</t>
+  </si>
+  <si>
+    <t>Review configs (standards, tool restriction, structured output) are a tested objective; see code.claude.com/docs/en/code-review</t>
+  </si>
+  <si>
+    <t>Lab 4: Memory hierarchy walk + skill triggering</t>
+  </si>
+  <si>
+    <t>Lab 5: Enforcement, not exhortation (highest-yield lab in the kit)</t>
+  </si>
+  <si>
+    <t>Lab 6: Headless CI with generator/reviewer isolation</t>
+  </si>
+  <si>
+    <t>Courses: Claude Code in Action; Intro to Agent Skills; Intro to Subagents</t>
+  </si>
+  <si>
+    <t>Academy - course catalog</t>
+  </si>
+  <si>
+    <t>Docs: GitHub Actions integration (CI scenario)</t>
+  </si>
+  <si>
+    <t>Code docs - GitHub Actions</t>
+  </si>
+  <si>
+    <t>Re-drill D3; must hold 5/5</t>
+  </si>
+  <si>
+    <t>P4 - D4 Prompt Eng &amp; Output</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>Baseline drill: D4 filter, 5 questions</t>
+  </si>
+  <si>
+    <t>Study Prompting best practices end to end (examples, chaining, agentic prompting)</t>
+  </si>
+  <si>
+    <t>Docs - Prompting best practices</t>
+  </si>
+  <si>
+    <t>Study Structured outputs; memorize: citations+format=400, prefill incompatible, format change kills cache, strict+JSON combinable</t>
+  </si>
+  <si>
+    <t>Docs - Structured outputs</t>
+  </si>
+  <si>
+    <t>Also covers extraction-schema design with optional/nullable fields and enums (tested objective)</t>
+  </si>
+  <si>
+    <t>Lab 1: Break JSON on purpose, then make it unbreakable</t>
+  </si>
+  <si>
+    <t>Lab 2: Strict tool use and schema drift</t>
+  </si>
+  <si>
+    <t>Lab 3: Validation-retry loop and example diversity</t>
+  </si>
+  <si>
+    <t>Hands-on with Console prompting tools: generator, improver, evaluation</t>
+  </si>
+  <si>
+    <t>Docs - Console prompting tools</t>
+  </si>
+  <si>
+    <t>Course: Building with the Claude API (find in Academy catalog)</t>
+  </si>
+  <si>
+    <t>Re-drill D4; must hold 5/5</t>
+  </si>
+  <si>
+    <t>P5 - D5 Context &amp; Reliability</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>Baseline drill: D5 filter, 5 questions</t>
+  </si>
+  <si>
+    <t>Docs: Context editing - tool-result clearing, thinking clearing, compaction summary structure</t>
+  </si>
+  <si>
+    <t>Docs - Context editing</t>
+  </si>
+  <si>
+    <t>Extra reading: joeyyu23.github.io/claude-code-handbook (architect / harness engineering)</t>
+  </si>
+  <si>
+    <t>Read: Effective context engineering for AI agents (engineering post)</t>
+  </si>
+  <si>
+    <t>Lab 7: Prompt caching forensics (prefix invalidation signatures)</t>
+  </si>
+  <si>
+    <t>Lab 8: Context editing under tool-call load</t>
+  </si>
+  <si>
+    <t>Lab 9: stop_reason handling + compaction contract</t>
+  </si>
+  <si>
+    <t>Docs: Batch processing - sync vs batch decision, custom_id, 24h window</t>
+  </si>
+  <si>
+    <t>Docs - Batch processing</t>
+  </si>
+  <si>
+    <t>Re-drill D5; must hold 5/5</t>
+  </si>
+  <si>
+    <t>P6 - Final Prep</t>
+  </si>
+  <si>
+    <t>Review 12-week repo: Key Anti-Patterns and Decision Frameworks tables</t>
+  </si>
+  <si>
+    <t>Community</t>
+  </si>
+  <si>
+    <t>GitHub - SGridworks 12-week program</t>
+  </si>
+  <si>
+    <t>Unofficial; when it disagrees with the docs, the docs win</t>
+  </si>
+  <si>
+    <t>Full 25-question honeypot drill, shuffled, cold; target 21+</t>
+  </si>
+  <si>
+    <t>Community mock: 60-question simulator (unofficial; pattern practice only)</t>
+  </si>
+  <si>
+    <t>Practice</t>
+  </si>
+  <si>
+    <t>anthropiccertifications.com</t>
+  </si>
+  <si>
+    <t>12-week repo practice tests (110 questions in practice-tests/)</t>
+  </si>
+  <si>
+    <t>GitHub - repo practice-tests folder</t>
+  </si>
+  <si>
+    <t>Official Skilljar practice exam, final pass; read EVERY rationale incl. correct answers</t>
+  </si>
+  <si>
+    <t>Day before: exam-strategy one-pager + terminology hit list; no new material</t>
+  </si>
+  <si>
+    <t>CCA-F Prep Dashboard</t>
+  </si>
+  <si>
+    <t>Overall progress</t>
+  </si>
+  <si>
+    <t>Hours remaining</t>
+  </si>
+  <si>
+    <t>Progress by phase</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Progress</t>
+  </si>
+  <si>
+    <t>Progress by domain</t>
+  </si>
+  <si>
+    <t>Exam weight</t>
+  </si>
+  <si>
+    <t>D1 - Agentic Architecture &amp; Orchestration</t>
+  </si>
+  <si>
+    <t>D2 - Tool Design &amp; MCP Integration</t>
+  </si>
+  <si>
+    <t>D3 - Claude Code Config &amp; Workflows</t>
+  </si>
+  <si>
+    <t>D4 - Prompt Eng &amp; Structured Output</t>
+  </si>
+  <si>
+    <t>D5 - Context Mgmt &amp; Reliability</t>
+  </si>
+  <si>
+    <t>Cross-domain (orient + final prep)</t>
+  </si>
+  <si>
+    <t>How to use</t>
+  </si>
+  <si>
+    <t>1. Work the Checklist tab top to bottom: P0 orientation, then one domain phase at a time (D1 through D5, ordered by domain number), then P6 final prep.</t>
+  </si>
+  <si>
+    <t>2. Edit ONLY the three input columns: Status (dropdown), Date done, and Notes. Every other cell, and this dashboard, is formula-driven.</t>
+  </si>
+  <si>
+    <t>3. Example entry: when you finish a task, set Status = Done and Date done = 2026-07-15 (any date format works); the row tints green and the Dashboard updates.</t>
+  </si>
+  <si>
+    <t>4. Status colors: green = Done, amber = In Progress. Red priority text = HIGH.</t>
+  </si>
+  <si>
+    <t>5. Resource links open docs and courses online; drill, labs, and strategy links open local files in this kit (keep the workbook in the kit's root folder).</t>
+  </si>
+  <si>
+    <t>6. Lab answer keys live in 03-Hands-On-Labs/_AnswerKeys/ - attempt each lab before opening its key.</t>
+  </si>
+  <si>
+    <t>Exam objective coverage map</t>
+  </si>
+  <si>
+    <t>Test objectives from the official exam blueprint (as reported section-wise on score reports). Each objective is mapped to where this kit covers it; doc coverage verified against the linked pages (July 2026).</t>
+  </si>
+  <si>
+    <t>Exam objective</t>
+  </si>
+  <si>
+    <t>Covered in this kit by</t>
+  </si>
+  <si>
+    <t>Primary reference (click to open)</t>
+  </si>
+  <si>
+    <t>Configure agentic loops to emit multiple tool calls within a single response turn, enabling parallel execution of independent subtasks and reducing total round-trip latency.</t>
+  </si>
+  <si>
+    <t>Lab 11 step 4 - Lab 14 step 3 - Drill Q16</t>
+  </si>
+  <si>
+    <t>Tool use overview</t>
+  </si>
+  <si>
+    <t>Apply session resumption techniques - including targeted re-analysis of changed files and context injection - to restore agent state accurately without repeating prior work.</t>
+  </si>
+  <si>
+    <t>Checklist P3 Sessions row - Strategy sheet 'State persistence'</t>
+  </si>
+  <si>
+    <t>Sessions</t>
+  </si>
+  <si>
+    <t>Construct subagent prompts that include all findings, structured data, and source metadata required for task completion without returning to the coordinator for missing context.</t>
+  </si>
+  <si>
+    <t>Lab 10 steps 1-2 - Drill Q17</t>
+  </si>
+  <si>
+    <t>How we built our multi-agent research system</t>
+  </si>
+  <si>
+    <t>Evaluate subagent delegation strategies - goal-oriented versus procedural instructions - and select the approach that enables adaptive behavior while maintaining coordinator visibility and control.</t>
+  </si>
+  <si>
+    <t>Strategy sheet 'Multi-agent' (delegation style)</t>
+  </si>
+  <si>
+    <t>Multi-agent research post ('Teach the orchestrator how to delegate')</t>
+  </si>
+  <si>
+    <t>Configure subagent invocations with appropriate tool restrictions, context scoping, and system prompts that constrain each agent to its designated role.</t>
+  </si>
+  <si>
+    <t>Lab 10 - Lab 14 - Drill Q23</t>
+  </si>
+  <si>
+    <t>Subagents in Claude Code</t>
+  </si>
+  <si>
+    <t>Diagnose misconfigured subagent spawning by identifying missing tool permissions, incorrect AgentDefinition parameters, or absent coordinator-to-subagent wiring.</t>
+  </si>
+  <si>
+    <t>Official links index (D1 section)</t>
+  </si>
+  <si>
+    <t>Subagents in the Agent SDK</t>
+  </si>
+  <si>
+    <t>Decompose complex tasks into dynamically generated subtasks that adapt as new information is discovered, rather than executing a fixed sequence regardless of intermediate findings.</t>
+  </si>
+  <si>
+    <t>Drill Q18 - Lab 10</t>
+  </si>
+  <si>
+    <t>Building effective agents (orchestrator-workers)</t>
+  </si>
+  <si>
+    <t>Select the appropriate agentic review architecture - plan mode, direct execution, or multi-phase workflow - based on task scope, risk level, and human approval requirements.</t>
+  </si>
+  <si>
+    <t>Checklist P3 Permission-modes row - Strategy sheet 'Review architecture'</t>
+  </si>
+  <si>
+    <t>Permission modes (incl. plan mode)</t>
+  </si>
+  <si>
+    <t>Design state persistence strategies for multi-agent pipelines that enable reliable resumption after interruption without repeating completed work or losing prior findings.</t>
+  </si>
+  <si>
+    <t>Drill Q19 - Strategy sheet 'State persistence'</t>
+  </si>
+  <si>
+    <t>Multi-agent research post (checkpoints, resume-on-error)</t>
+  </si>
+  <si>
+    <t>Evaluate multi-agent orchestration patterns - coordinator-worker, parallel execution, and sequential pipelines - to select the structure best satisfying research coverage, latency, and reliability requirements.</t>
+  </si>
+  <si>
+    <t>Building effective agents (the five workflow patterns)</t>
+  </si>
+  <si>
+    <t>Configure Claude Code CLI invocations for automated CI/CD pipelines using non-interactive flags, permission modes, and cost and turn limits that prevent runaway executions.</t>
+  </si>
+  <si>
+    <t>Lab 6 - Drill Q9 - Strategy sheet field note (--bare)</t>
+  </si>
+  <si>
+    <t>CLI reference + Headless</t>
+  </si>
+  <si>
+    <t>Structure iterative refinement workflows by providing concrete input-output examples, targeted feedback on specific failures, and batched issue descriptions for consolidated evaluation.</t>
+  </si>
+  <si>
+    <t>Lab 3 (validation-retry, targeted feedback)</t>
+  </si>
+  <si>
+    <t>Prompting best practices</t>
+  </si>
+  <si>
+    <t>Design Claude Code review configurations that load the correct project standards, restrict unnecessary tool access, and produce structured output suitable for automated downstream processing.</t>
+  </si>
+  <si>
+    <t>Lab 6 (two-stage pipeline) - Checklist P3 Sessions/Code-review row</t>
+  </si>
+  <si>
+    <t>Code review</t>
+  </si>
+  <si>
+    <t>Apply the context: fork frontmatter option to Skill and slash command configurations that should execute in an isolated subagent context, preventing cross-contamination of session state.</t>
+  </si>
+  <si>
+    <t>Strategy sheet 'Slash command vs skill vs subagent' - Checklist P3 Skills row</t>
+  </si>
+  <si>
+    <t>Skills ('Run skills in a subagent')</t>
+  </si>
+  <si>
+    <t>Improve automated test generation quality by providing existing test files as context, defining fixture conventions, and specifying criteria that distinguish meaningful behavioral tests from trivial assertions.</t>
+  </si>
+  <si>
+    <t>Checklist P3 Tools-reference/Common-workflows row</t>
+  </si>
+  <si>
+    <t>Common workflows (testing)</t>
+  </si>
+  <si>
+    <t>Select the correct Claude Code configuration mechanism - CLAUDE.md, .claude/rules/ with glob patterns, Skills, hooks, or settings permissions - based on guidance type and when it should apply.</t>
+  </si>
+  <si>
+    <t>Labs 4-5 - Drill Q6-Q8, Q10 - Strategy sheet 'Config mechanism selection'</t>
+  </si>
+  <si>
+    <t>Extend Claude Code</t>
+  </si>
+  <si>
+    <t>Apply systematic codebase exploration strategies using Grep, Glob, and Read tools that build incremental understanding while managing context window constraints.</t>
+  </si>
+  <si>
+    <t>Strategy sheet 'Built-in tool selection'</t>
+  </si>
+  <si>
+    <t>Common workflows + Tools reference</t>
+  </si>
+  <si>
+    <t>Design subagent output schemas that render structured data, prose summaries, and citation metadata in the format best suited to downstream synthesis and reporting.</t>
+  </si>
+  <si>
+    <t>Lab 10 (Finding schema)</t>
+  </si>
+  <si>
+    <t>Multi-agent research post (appendix: subagent outputs)</t>
+  </si>
+  <si>
+    <t>Design synthesis agent behavior that preserves source-level uncertainty, distinguishing well-established findings from contested claims rather than collapsing conflicting data into single confident statements.</t>
+  </si>
+  <si>
+    <t>Lab 10 step 4 (provenance) - Drill Q14</t>
+  </si>
+  <si>
+    <t>Multi-agent research post</t>
+  </si>
+  <si>
+    <t>Apply context management strategies - subagent isolation, scratchpad files, and targeted file reading - to sustain coherent codebase exploration across sessions exceeding context limits.</t>
+  </si>
+  <si>
+    <t>Lab 8 - Lab 10 (isolation)</t>
+  </si>
+  <si>
+    <t>Effective context engineering for AI agents</t>
+  </si>
+  <si>
+    <t>Apply context window optimization techniques - summarization, sliding windows, structured state objects, and selective retention - to maintain response quality as conversations exceed practical token limits.</t>
+  </si>
+  <si>
+    <t>Labs 8-9 - Drill Q11, Q15</t>
+  </si>
+  <si>
+    <t>Context editing</t>
+  </si>
+  <si>
+    <t>Design human review routing strategies that direct extractions to reviewers based on confidence scores, document characteristics, and field-level ambiguity rather than random sampling.</t>
+  </si>
+  <si>
+    <t>Strategy sheet 'Human review routing' - Lab 12 part 3 (signal quality)</t>
+  </si>
+  <si>
+    <t>Exam-day one-pager</t>
+  </si>
+  <si>
+    <t>Select the appropriate API processing mode - synchronous Messages API or asynchronous Message Batches API - based on latency requirements, workflow blocking behavior, and acceptable processing windows.</t>
+  </si>
+  <si>
+    <t>Checklist P5 Batch row - Strategy sheet 'Headless / CI'</t>
+  </si>
+  <si>
+    <t>Batch processing</t>
+  </si>
+  <si>
+    <t>Design specialized review passes that separate concerns - security, business logic, API design - into focused prompts with dedicated few-shot examples, preventing recall trade-offs from competing concerns in a single prompt.</t>
+  </si>
+  <si>
+    <t>Strategy sheet 'Review architecture' - Drill Q5</t>
+  </si>
+  <si>
+    <t>Select and implement the most reliable structured output method - tool use with JSON schema, prompt-based formatting, or prefilled responses - based on required schema compliance strictness.</t>
+  </si>
+  <si>
+    <t>Lab 1 - Drill Q1</t>
+  </si>
+  <si>
+    <t>Structured outputs</t>
+  </si>
+  <si>
+    <t>Design extraction schemas with optional fields, nullable values, and appropriate enum definitions that allow the model to accurately represent missing or ambiguous information without fabricating values.</t>
+  </si>
+  <si>
+    <t>Lab 2 - Checklist P4 Structured-outputs row</t>
+  </si>
+  <si>
+    <t>Implement tool use with defined JSON schemas to enforce structured output compliance, and configure tool_choice to guarantee tool invocation when conversational responses would cause downstream failures.</t>
+  </si>
+  <si>
+    <t>Lab 13 - Drill Q22</t>
+  </si>
+  <si>
+    <t>Resolve structured output truncation failures by splitting large review tasks into smaller scoped API calls and merging resulting data structures, rather than increasing max_tokens beyond practical limits.</t>
+  </si>
+  <si>
+    <t>Lab 9 - Drill Q13 - Strategy sheet 'stop_reason' (split-and-merge)</t>
+  </si>
+  <si>
+    <t>Apply extraction accuracy patterns - structured schemas with optional fields, format normalization instructions, and few-shot examples - to reduce hallucination and improve consistency across varied document formats.</t>
+  </si>
+  <si>
+    <t>Labs 1-3</t>
+  </si>
+  <si>
+    <t>Structured outputs + Prompting best practices</t>
+  </si>
+  <si>
+    <t>Reduce automated review false positive rates by supplying project-specific conventions, accepted patterns, and exclusion criteria as persistent context applied on every review.</t>
+  </si>
+  <si>
+    <t>Lab 4 (CLAUDE.md) - Checklist P3 Memory row</t>
+  </si>
+  <si>
+    <t>Memory + Code review</t>
+  </si>
+  <si>
+    <t>Design prompt criteria that define explicit inclusion and exclusion boundaries, preventing the model from generating findings or extractions in categories where performance is unreliable.</t>
+  </si>
+  <si>
+    <t>Lab 3</t>
+  </si>
+  <si>
+    <t>Select the appropriate Claude Code built-in tool - Grep, Glob, Read, or Bash - based on the nature of the search or file operation required for a given codebase task.</t>
+  </si>
+  <si>
+    <t>Tools reference</t>
+  </si>
+  <si>
+    <t>Configure tool distribution in multi-agent systems by assigning each subagent only the tools required for its designated role, reducing decision complexity and preventing out-of-role tool invocations.</t>
+  </si>
+  <si>
+    <t>Lab 14 - Drill Q23</t>
+  </si>
+  <si>
+    <t>Subagents + Tool use overview</t>
+  </si>
+  <si>
+    <t>Distinguish between MCP resources and tools, and expose server content as resources to reduce exploratory tool calls and improve agent efficiency in cross-system queries.</t>
+  </si>
+  <si>
+    <t>Drill Q24 - Lab 15</t>
+  </si>
+  <si>
+    <t>Model Context Protocol docs</t>
+  </si>
+  <si>
+    <t>Integrate MCP servers into Claude Code and agent applications by selecting the correct server scope, configuring authentication via environment variable expansion, and verifying tool discovery.</t>
+  </si>
+  <si>
+    <t>Lab 15 - Drill Q25</t>
+  </si>
+  <si>
+    <t>MCP in Claude Code</t>
+  </si>
+  <si>
+    <t>Write MCP tool descriptions that clearly distinguish each tool's purpose, input formats, use-case boundaries, and relationships to semantically similar tools, reducing misrouting and incorrect tool selection.</t>
+  </si>
+  <si>
+    <t>Lab 13 - Drill Q21</t>
+  </si>
+  <si>
+    <t>Tool use overview + MCP docs</t>
+  </si>
+  <si>
+    <t>Configure the tool_choice parameter to guarantee tool invocation when structured output is required, and sequence multi-tool workflows so prerequisite data is obtained before dependent tools are called.</t>
+  </si>
+  <si>
+    <t>Lab 13 step 2 - Drill Q22</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0%"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -871,54 +885,34 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="10"/>
       <color rgb="FF0563C1"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="14"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -937,14 +931,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFC9CFD8"/>
       </left>
@@ -960,138 +954,53 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="15">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="3">
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F3864"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
+      <font>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFA83240"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFA83240"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0563C1"/>
-          <bgColor rgb="FF000000"/>
+        <patternFill>
+          <bgColor rgb="FFFFF3D2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1102,24 +1011,8 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF3D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <charset val="1"/>
-        <family val="0"/>
-        <b val="1"/>
-        <color rgb="FFA83240"/>
-        <sz val="10"/>
-      </font>
-    </dxf>
   </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1178,21 +1071,29 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1234,12 +1135,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -1268,7 +1169,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1289,7 +1190,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1340,7 +1241,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1358,34 +1259,33 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K61"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="52"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="4" customWidth="1"/>
+    <col min="3" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="74" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="34" customWidth="1"/>
+    <col min="8" max="8" width="7" customWidth="1"/>
+    <col min="9" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1420,11 +1320,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1442,7 +1342,7 @@
       <c r="G2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="3">
         <v>0.3</v>
       </c>
       <c r="I2" s="3" t="s">
@@ -1451,11 +1351,11 @@
       <c r="J2" s="3"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="3">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -1473,7 +1373,7 @@
       <c r="G3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="3">
         <v>1.5</v>
       </c>
       <c r="I3" s="3" t="s">
@@ -1484,11 +1384,11 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="3">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -1506,7 +1406,7 @@
       <c r="G4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="3">
         <v>0.3</v>
       </c>
       <c r="I4" s="3" t="s">
@@ -1517,11 +1417,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="3">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -1539,7 +1439,7 @@
       <c r="G5" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="3">
         <v>0.4</v>
       </c>
       <c r="I5" s="3" t="s">
@@ -1548,11 +1448,11 @@
       <c r="J5" s="3"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="3">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -1570,7 +1470,7 @@
       <c r="G6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H6" s="3">
         <v>0.8</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -1581,11 +1481,11 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:11" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="3">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -1603,7 +1503,7 @@
       <c r="G7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="3">
         <v>0.8</v>
       </c>
       <c r="I7" s="3" t="s">
@@ -1614,11 +1514,11 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="3">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -1636,7 +1536,7 @@
       <c r="G8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" s="3">
         <v>0.8</v>
       </c>
       <c r="I8" s="3" t="s">
@@ -1647,11 +1547,11 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="3">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
@@ -1669,7 +1569,7 @@
       <c r="G9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" s="3">
         <v>0.5</v>
       </c>
       <c r="I9" s="3" t="s">
@@ -1680,11 +1580,11 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="3">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1702,7 +1602,7 @@
       <c r="G10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="3">
         <v>0.8</v>
       </c>
       <c r="I10" s="3" t="s">
@@ -1711,11 +1611,11 @@
       <c r="J10" s="3"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="3">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1733,7 +1633,7 @@
       <c r="G11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" s="3">
         <v>0.7</v>
       </c>
       <c r="I11" s="3" t="s">
@@ -1742,11 +1642,11 @@
       <c r="J11" s="3"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="3">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -1764,7 +1664,7 @@
       <c r="G12" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="H12" s="3">
         <v>0.7</v>
       </c>
       <c r="I12" s="3" t="s">
@@ -1773,11 +1673,11 @@
       <c r="J12" s="3"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="3">
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
@@ -1795,7 +1695,7 @@
       <c r="G13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="H13" s="3">
         <v>0.3</v>
       </c>
       <c r="I13" s="3" t="s">
@@ -1804,11 +1704,11 @@
       <c r="J13" s="3"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="3">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -1826,7 +1726,7 @@
       <c r="G14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="H14" s="3">
         <v>0.4</v>
       </c>
       <c r="I14" s="3" t="s">
@@ -1835,11 +1735,11 @@
       <c r="J14" s="3"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="3">
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
@@ -1857,7 +1757,7 @@
       <c r="G15" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="H15" s="3">
         <v>0.8</v>
       </c>
       <c r="I15" s="3" t="s">
@@ -1868,11 +1768,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="3">
         <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
@@ -1890,7 +1790,7 @@
       <c r="G16" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H16" s="3" t="n">
+      <c r="H16" s="3">
         <v>0.7</v>
       </c>
       <c r="I16" s="3" t="s">
@@ -1901,11 +1801,11 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="3">
         <v>16</v>
       </c>
       <c r="C17" s="3" t="s">
@@ -1923,7 +1823,7 @@
       <c r="G17" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="H17" s="3" t="n">
+      <c r="H17" s="3">
         <v>1.5</v>
       </c>
       <c r="I17" s="3" t="s">
@@ -1932,11 +1832,11 @@
       <c r="J17" s="3"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="3">
         <v>17</v>
       </c>
       <c r="C18" s="3" t="s">
@@ -1954,7 +1854,7 @@
       <c r="G18" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H18" s="3" t="n">
+      <c r="H18" s="3">
         <v>0.6</v>
       </c>
       <c r="I18" s="3" t="s">
@@ -1963,11 +1863,11 @@
       <c r="J18" s="3"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="3">
         <v>18</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -1985,7 +1885,7 @@
       <c r="G19" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H19" s="3" t="n">
+      <c r="H19" s="3">
         <v>0.6</v>
       </c>
       <c r="I19" s="3" t="s">
@@ -1994,11 +1894,11 @@
       <c r="J19" s="3"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="3">
         <v>19</v>
       </c>
       <c r="C20" s="3" t="s">
@@ -2016,7 +1916,7 @@
       <c r="G20" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H20" s="3" t="n">
+      <c r="H20" s="3">
         <v>0.7</v>
       </c>
       <c r="I20" s="3" t="s">
@@ -2025,11 +1925,11 @@
       <c r="J20" s="3"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="3">
         <v>20</v>
       </c>
       <c r="C21" s="3" t="s">
@@ -2047,7 +1947,7 @@
       <c r="G21" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="H21" s="3">
         <v>0.3</v>
       </c>
       <c r="I21" s="3" t="s">
@@ -2056,11 +1956,11 @@
       <c r="J21" s="3"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="3">
         <v>21</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -2078,7 +1978,7 @@
       <c r="G22" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="3" t="n">
+      <c r="H22" s="3">
         <v>0.4</v>
       </c>
       <c r="I22" s="3" t="s">
@@ -2087,11 +1987,11 @@
       <c r="J22" s="3"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="3">
         <v>22</v>
       </c>
       <c r="C23" s="3" t="s">
@@ -2109,7 +2009,7 @@
       <c r="G23" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H23" s="3" t="n">
+      <c r="H23" s="3">
         <v>0.5</v>
       </c>
       <c r="I23" s="3" t="s">
@@ -2120,11 +2020,11 @@
         <v>70</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="3">
         <v>23</v>
       </c>
       <c r="C24" s="3" t="s">
@@ -2142,7 +2042,7 @@
       <c r="G24" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="3" t="n">
+      <c r="H24" s="3">
         <v>0.8</v>
       </c>
       <c r="I24" s="3" t="s">
@@ -2153,11 +2053,11 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="3">
         <v>24</v>
       </c>
       <c r="C25" s="3" t="s">
@@ -2175,7 +2075,7 @@
       <c r="G25" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="H25" s="3" t="n">
+      <c r="H25" s="3">
         <v>0.8</v>
       </c>
       <c r="I25" s="3" t="s">
@@ -2184,11 +2084,11 @@
       <c r="J25" s="3"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="3">
         <v>25</v>
       </c>
       <c r="C26" s="3" t="s">
@@ -2206,7 +2106,7 @@
       <c r="G26" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="H26" s="3" t="n">
+      <c r="H26" s="3">
         <v>0.7</v>
       </c>
       <c r="I26" s="3" t="s">
@@ -2217,11 +2117,11 @@
         <v>78</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="3">
         <v>26</v>
       </c>
       <c r="C27" s="3" t="s">
@@ -2239,7 +2139,7 @@
       <c r="G27" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="H27" s="3" t="n">
+      <c r="H27" s="3">
         <v>0.4</v>
       </c>
       <c r="I27" s="3" t="s">
@@ -2248,11 +2148,11 @@
       <c r="J27" s="3"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="3">
         <v>27</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -2270,7 +2170,7 @@
       <c r="G28" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="H28" s="3" t="n">
+      <c r="H28" s="3">
         <v>0.6</v>
       </c>
       <c r="I28" s="3" t="s">
@@ -2281,11 +2181,11 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B29" s="3">
         <v>28</v>
       </c>
       <c r="C29" s="3" t="s">
@@ -2303,7 +2203,7 @@
       <c r="G29" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="H29" s="3" t="n">
+      <c r="H29" s="3">
         <v>0.5</v>
       </c>
       <c r="I29" s="3" t="s">
@@ -2314,11 +2214,11 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:11" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="3">
         <v>29</v>
       </c>
       <c r="C30" s="3" t="s">
@@ -2336,7 +2236,7 @@
       <c r="G30" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="H30" s="3" t="n">
+      <c r="H30" s="3">
         <v>0.6</v>
       </c>
       <c r="I30" s="3" t="s">
@@ -2347,11 +2247,11 @@
         <v>89</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:11" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="3">
         <v>30</v>
       </c>
       <c r="C31" s="3" t="s">
@@ -2369,7 +2269,7 @@
       <c r="G31" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="H31" s="3" t="n">
+      <c r="H31" s="3">
         <v>0.7</v>
       </c>
       <c r="I31" s="3" t="s">
@@ -2380,11 +2280,11 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:11" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="3">
         <v>31</v>
       </c>
       <c r="C32" s="3" t="s">
@@ -2402,7 +2302,7 @@
       <c r="G32" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="H32" s="3" t="n">
+      <c r="H32" s="3">
         <v>0.5</v>
       </c>
       <c r="I32" s="3" t="s">
@@ -2413,11 +2313,11 @@
         <v>95</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="3">
         <v>32</v>
       </c>
       <c r="C33" s="3" t="s">
@@ -2435,7 +2335,7 @@
       <c r="G33" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H33" s="3" t="n">
+      <c r="H33" s="3">
         <v>0.7</v>
       </c>
       <c r="I33" s="3" t="s">
@@ -2444,11 +2344,11 @@
       <c r="J33" s="3"/>
       <c r="K33" s="2"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="3">
         <v>33</v>
       </c>
       <c r="C34" s="3" t="s">
@@ -2466,7 +2366,7 @@
       <c r="G34" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H34" s="3" t="n">
+      <c r="H34" s="3">
         <v>0.7</v>
       </c>
       <c r="I34" s="3" t="s">
@@ -2475,11 +2375,11 @@
       <c r="J34" s="3"/>
       <c r="K34" s="2"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="3">
         <v>34</v>
       </c>
       <c r="C35" s="3" t="s">
@@ -2497,7 +2397,7 @@
       <c r="G35" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H35" s="3" t="n">
+      <c r="H35" s="3">
         <v>0.8</v>
       </c>
       <c r="I35" s="3" t="s">
@@ -2506,11 +2406,11 @@
       <c r="J35" s="3"/>
       <c r="K35" s="2"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B36" s="3">
         <v>35</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -2528,7 +2428,7 @@
       <c r="G36" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="H36" s="3" t="n">
+      <c r="H36" s="3">
         <v>2.5</v>
       </c>
       <c r="I36" s="3" t="s">
@@ -2537,11 +2437,11 @@
       <c r="J36" s="3"/>
       <c r="K36" s="2"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B37" s="3">
         <v>36</v>
       </c>
       <c r="C37" s="3" t="s">
@@ -2559,7 +2459,7 @@
       <c r="G37" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="H37" s="3" t="n">
+      <c r="H37" s="3">
         <v>0.4</v>
       </c>
       <c r="I37" s="3" t="s">
@@ -2568,11 +2468,11 @@
       <c r="J37" s="3"/>
       <c r="K37" s="2"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="3">
         <v>37</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -2590,7 +2490,7 @@
       <c r="G38" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H38" s="3" t="n">
+      <c r="H38" s="3">
         <v>0.3</v>
       </c>
       <c r="I38" s="3" t="s">
@@ -2599,11 +2499,11 @@
       <c r="J38" s="3"/>
       <c r="K38" s="2"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B39" s="3">
         <v>38</v>
       </c>
       <c r="C39" s="3" t="s">
@@ -2621,7 +2521,7 @@
       <c r="G39" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H39" s="3" t="n">
+      <c r="H39" s="3">
         <v>0.4</v>
       </c>
       <c r="I39" s="3" t="s">
@@ -2630,11 +2530,11 @@
       <c r="J39" s="3"/>
       <c r="K39" s="2"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="3">
         <v>39</v>
       </c>
       <c r="C40" s="3" t="s">
@@ -2652,7 +2552,7 @@
       <c r="G40" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="H40" s="3" t="n">
+      <c r="H40" s="3">
         <v>1.2</v>
       </c>
       <c r="I40" s="3" t="s">
@@ -2661,11 +2561,11 @@
       <c r="J40" s="3"/>
       <c r="K40" s="2"/>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B41" s="3">
         <v>40</v>
       </c>
       <c r="C41" s="3" t="s">
@@ -2683,7 +2583,7 @@
       <c r="G41" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="H41" s="3" t="n">
+      <c r="H41" s="3">
         <v>1</v>
       </c>
       <c r="I41" s="3" t="s">
@@ -2694,11 +2594,11 @@
         <v>111</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B42" s="3">
         <v>41</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -2716,7 +2616,7 @@
       <c r="G42" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H42" s="3" t="n">
+      <c r="H42" s="3">
         <v>0.7</v>
       </c>
       <c r="I42" s="3" t="s">
@@ -2725,11 +2625,11 @@
       <c r="J42" s="3"/>
       <c r="K42" s="2"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B43" s="3">
         <v>42</v>
       </c>
       <c r="C43" s="3" t="s">
@@ -2747,7 +2647,7 @@
       <c r="G43" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H43" s="3" t="n">
+      <c r="H43" s="3">
         <v>0.5</v>
       </c>
       <c r="I43" s="3" t="s">
@@ -2756,11 +2656,11 @@
       <c r="J43" s="3"/>
       <c r="K43" s="2"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B44" s="3">
         <v>43</v>
       </c>
       <c r="C44" s="3" t="s">
@@ -2778,7 +2678,7 @@
       <c r="G44" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H44" s="3" t="n">
+      <c r="H44" s="3">
         <v>0.8</v>
       </c>
       <c r="I44" s="3" t="s">
@@ -2787,11 +2687,11 @@
       <c r="J44" s="3"/>
       <c r="K44" s="2"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B45" s="3">
         <v>44</v>
       </c>
       <c r="C45" s="3" t="s">
@@ -2809,7 +2709,7 @@
       <c r="G45" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="H45" s="3" t="n">
+      <c r="H45" s="3">
         <v>0.5</v>
       </c>
       <c r="I45" s="3" t="s">
@@ -2818,11 +2718,11 @@
       <c r="J45" s="3"/>
       <c r="K45" s="2"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B46" s="3">
         <v>45</v>
       </c>
       <c r="C46" s="3" t="s">
@@ -2840,7 +2740,7 @@
       <c r="G46" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="H46" s="3" t="n">
+      <c r="H46" s="3">
         <v>2</v>
       </c>
       <c r="I46" s="3" t="s">
@@ -2849,11 +2749,11 @@
       <c r="J46" s="3"/>
       <c r="K46" s="2"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B47" s="3" t="n">
+      <c r="B47" s="3">
         <v>46</v>
       </c>
       <c r="C47" s="3" t="s">
@@ -2871,7 +2771,7 @@
       <c r="G47" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H47" s="3" t="n">
+      <c r="H47" s="3">
         <v>0.3</v>
       </c>
       <c r="I47" s="3" t="s">
@@ -2880,11 +2780,11 @@
       <c r="J47" s="3"/>
       <c r="K47" s="2"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B48" s="3">
         <v>47</v>
       </c>
       <c r="C48" s="3" t="s">
@@ -2902,7 +2802,7 @@
       <c r="G48" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H48" s="3" t="n">
+      <c r="H48" s="3">
         <v>0.4</v>
       </c>
       <c r="I48" s="3" t="s">
@@ -2911,11 +2811,11 @@
       <c r="J48" s="3"/>
       <c r="K48" s="2"/>
     </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:11" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B49" s="3">
         <v>48</v>
       </c>
       <c r="C49" s="3" t="s">
@@ -2933,7 +2833,7 @@
       <c r="G49" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="H49" s="3" t="n">
+      <c r="H49" s="3">
         <v>0.9</v>
       </c>
       <c r="I49" s="3" t="s">
@@ -2944,11 +2844,11 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B50" s="3" t="n">
+      <c r="B50" s="3">
         <v>49</v>
       </c>
       <c r="C50" s="3" t="s">
@@ -2966,7 +2866,7 @@
       <c r="G50" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H50" s="3" t="n">
+      <c r="H50" s="3">
         <v>0.7</v>
       </c>
       <c r="I50" s="3" t="s">
@@ -2975,11 +2875,11 @@
       <c r="J50" s="3"/>
       <c r="K50" s="2"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B51" s="3">
         <v>50</v>
       </c>
       <c r="C51" s="3" t="s">
@@ -2997,7 +2897,7 @@
       <c r="G51" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H51" s="3" t="n">
+      <c r="H51" s="3">
         <v>0.6</v>
       </c>
       <c r="I51" s="3" t="s">
@@ -3006,11 +2906,11 @@
       <c r="J51" s="3"/>
       <c r="K51" s="2"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B52" s="3" t="n">
+      <c r="B52" s="3">
         <v>51</v>
       </c>
       <c r="C52" s="3" t="s">
@@ -3028,7 +2928,7 @@
       <c r="G52" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H52" s="3" t="n">
+      <c r="H52" s="3">
         <v>0.8</v>
       </c>
       <c r="I52" s="3" t="s">
@@ -3037,11 +2937,11 @@
       <c r="J52" s="3"/>
       <c r="K52" s="2"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B53" s="3" t="n">
+      <c r="B53" s="3">
         <v>52</v>
       </c>
       <c r="C53" s="3" t="s">
@@ -3059,7 +2959,7 @@
       <c r="G53" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H53" s="3" t="n">
+      <c r="H53" s="3">
         <v>0.7</v>
       </c>
       <c r="I53" s="3" t="s">
@@ -3068,11 +2968,11 @@
       <c r="J53" s="3"/>
       <c r="K53" s="2"/>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B54" s="3" t="n">
+      <c r="B54" s="3">
         <v>53</v>
       </c>
       <c r="C54" s="3" t="s">
@@ -3090,7 +2990,7 @@
       <c r="G54" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="H54" s="3" t="n">
+      <c r="H54" s="3">
         <v>0.4</v>
       </c>
       <c r="I54" s="3" t="s">
@@ -3099,11 +2999,11 @@
       <c r="J54" s="3"/>
       <c r="K54" s="2"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="3" t="n">
+      <c r="B55" s="3">
         <v>54</v>
       </c>
       <c r="C55" s="3" t="s">
@@ -3121,7 +3021,7 @@
       <c r="G55" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H55" s="3" t="n">
+      <c r="H55" s="3">
         <v>0.3</v>
       </c>
       <c r="I55" s="3" t="s">
@@ -3130,11 +3030,11 @@
       <c r="J55" s="3"/>
       <c r="K55" s="2"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B56" s="3" t="n">
+      <c r="B56" s="3">
         <v>55</v>
       </c>
       <c r="C56" s="3" t="s">
@@ -3152,7 +3052,7 @@
       <c r="G56" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="H56" s="3" t="n">
+      <c r="H56" s="3">
         <v>0.5</v>
       </c>
       <c r="I56" s="3" t="s">
@@ -3163,11 +3063,11 @@
         <v>136</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B57" s="3" t="n">
+      <c r="B57" s="3">
         <v>56</v>
       </c>
       <c r="C57" s="3" t="s">
@@ -3185,7 +3085,7 @@
       <c r="G57" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H57" s="3" t="n">
+      <c r="H57" s="3">
         <v>0.8</v>
       </c>
       <c r="I57" s="3" t="s">
@@ -3194,11 +3094,11 @@
       <c r="J57" s="3"/>
       <c r="K57" s="2"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B58" s="3" t="n">
+      <c r="B58" s="3">
         <v>57</v>
       </c>
       <c r="C58" s="3" t="s">
@@ -3216,7 +3116,7 @@
       <c r="G58" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="H58" s="3" t="n">
+      <c r="H58" s="3">
         <v>2</v>
       </c>
       <c r="I58" s="3" t="s">
@@ -3225,11 +3125,11 @@
       <c r="J58" s="3"/>
       <c r="K58" s="2"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B59" s="3" t="n">
+      <c r="B59" s="3">
         <v>58</v>
       </c>
       <c r="C59" s="3" t="s">
@@ -3247,7 +3147,7 @@
       <c r="G59" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="H59" s="3" t="n">
+      <c r="H59" s="3">
         <v>2.5</v>
       </c>
       <c r="I59" s="3" t="s">
@@ -3256,11 +3156,11 @@
       <c r="J59" s="3"/>
       <c r="K59" s="2"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B60" s="3" t="n">
+      <c r="B60" s="3">
         <v>59</v>
       </c>
       <c r="C60" s="3" t="s">
@@ -3278,7 +3178,7 @@
       <c r="G60" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H60" s="3" t="n">
+      <c r="H60" s="3">
         <v>1.5</v>
       </c>
       <c r="I60" s="3" t="s">
@@ -3287,11 +3187,11 @@
       <c r="J60" s="3"/>
       <c r="K60" s="2"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B61" s="3" t="n">
+      <c r="B61" s="3">
         <v>60</v>
       </c>
       <c r="C61" s="3" t="s">
@@ -3309,7 +3209,7 @@
       <c r="G61" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H61" s="3" t="n">
+      <c r="H61" s="3">
         <v>0.5</v>
       </c>
       <c r="I61" s="3" t="s">
@@ -3319,141 +3219,132 @@
       <c r="K61" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K61"/>
+  <autoFilter ref="A1:K61" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A2:K61">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$I2="Done"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>$I2="In Progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C61">
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" dxfId="0" priority="4">
       <formula>$C2="HIGH"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Pick from the list: Not Started, In Progress, Done" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I61" type="list">
+    <dataValidation type="list" allowBlank="1" error="Pick from the list: Not Started, In Progress, Done" sqref="I2:I61" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In Progress,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" display="01 - Official links index"/>
-    <hyperlink ref="G3" r:id="rId2" display="Skilljar - CCA-F certification page"/>
-    <hyperlink ref="G4" r:id="rId3" display="05 - Exam-day one-pager"/>
-    <hyperlink ref="G5" r:id="rId4" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G6" r:id="rId5" display="Anthropic engineering post"/>
-    <hyperlink ref="G7" r:id="rId6" display="Anthropic engineering post"/>
-    <hyperlink ref="G8" r:id="rId7" display="Docs - Tool use overview"/>
-    <hyperlink ref="G9" r:id="rId8" display="Code docs - Subagents"/>
-    <hyperlink ref="G10" r:id="rId9" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G11" r:id="rId10" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G12" r:id="rId11" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G13" r:id="rId12" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G14" r:id="rId13" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G15" r:id="rId14" display="Docs - Tool use overview"/>
-    <hyperlink ref="G16" r:id="rId15" display="Code docs - MCP"/>
-    <hyperlink ref="G17" r:id="rId16" display="Academy - Intro to MCP"/>
-    <hyperlink ref="G18" r:id="rId17" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G19" r:id="rId18" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G20" r:id="rId19" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G21" r:id="rId20" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G22" r:id="rId21" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G23" r:id="rId22" display="Code docs - Extend Claude Code"/>
-    <hyperlink ref="G24" r:id="rId23" display="Code docs - Memory"/>
-    <hyperlink ref="G25" r:id="rId24" display="Code docs - Hooks"/>
-    <hyperlink ref="G26" r:id="rId25" display="Code docs - Skills"/>
-    <hyperlink ref="G27" r:id="rId26" display="Code docs - Slash commands"/>
-    <hyperlink ref="G28" r:id="rId27" display="Code docs - Settings"/>
-    <hyperlink ref="G29" r:id="rId28" display="Code docs - Permission modes"/>
-    <hyperlink ref="G30" r:id="rId29" display="Code docs - CLI reference"/>
-    <hyperlink ref="G31" r:id="rId30" display="Code docs - Tools reference"/>
-    <hyperlink ref="G32" r:id="rId31" display="Code docs - Sessions"/>
-    <hyperlink ref="G33" r:id="rId32" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G34" r:id="rId33" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G35" r:id="rId34" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G36" r:id="rId35" display="Academy - course catalog"/>
-    <hyperlink ref="G37" r:id="rId36" display="Code docs - GitHub Actions"/>
-    <hyperlink ref="G38" r:id="rId37" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G39" r:id="rId38" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G40" r:id="rId39" display="Docs - Prompting best practices"/>
-    <hyperlink ref="G41" r:id="rId40" display="Docs - Structured outputs"/>
-    <hyperlink ref="G42" r:id="rId41" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G43" r:id="rId42" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G44" r:id="rId43" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G45" r:id="rId44" display="Docs - Console prompting tools"/>
-    <hyperlink ref="G46" r:id="rId45" display="Academy - course catalog"/>
-    <hyperlink ref="G47" r:id="rId46" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G48" r:id="rId47" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G49" r:id="rId48" display="Docs - Context editing"/>
-    <hyperlink ref="G50" r:id="rId49" display="Anthropic engineering post"/>
-    <hyperlink ref="G51" r:id="rId50" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G52" r:id="rId51" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G53" r:id="rId52" display="03 - Labs index (domain-labs.md)"/>
-    <hyperlink ref="G54" r:id="rId53" display="Docs - Batch processing"/>
-    <hyperlink ref="G55" r:id="rId54" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G56" r:id="rId55" display="GitHub - SGridworks 12-week program"/>
-    <hyperlink ref="G57" r:id="rId56" display="02 - Honeypot drill (open in browser)"/>
-    <hyperlink ref="G58" r:id="rId57" display="anthropiccertifications.com"/>
-    <hyperlink ref="G59" r:id="rId58" display="GitHub - repo practice-tests folder"/>
-    <hyperlink ref="G60" r:id="rId59" display="Skilljar - CCA-F certification page"/>
-    <hyperlink ref="G61" r:id="rId60" display="05 - Exam-day one-pager"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="G6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="G7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="G8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="G9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="G10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="G11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="G12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="G13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="G14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="G15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="G16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="G17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="G18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="G19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="G20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="G21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="G22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="G23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="G24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="G25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="G26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="G27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="G28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="G29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="G30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="G31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="G32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="G33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="G34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="G35" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="G36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="G37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="G38" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="G39" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="G40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="G41" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="G42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="G43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="G44" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="G45" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="G46" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="G47" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="G48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="G49" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="G50" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="G51" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="G52" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="G53" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="G54" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="G55" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="G56" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="G57" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="G58" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="G59" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="G60" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="G61" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId61"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col min="1" max="1" width="78" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" ht="17.649999999999999" x14ac:dyDescent="0.5">
       <c r="A1" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="B3" s="7" t="n">
-        <f aca="false">COUNTIF(Checklist!$I$2:$I$61,"Done")/60</f>
+      <c r="B3" s="7">
+        <f>COUNTIF(Checklist!$I$2:$I$61,"Done")/60</f>
         <v>0</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="D3" s="8" t="n">
-        <f aca="false">SUMIFS(Checklist!$H$2:$H$61,Checklist!$I$2:$I$61,"&lt;&gt;Done")</f>
-        <v>45.4</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D3" s="8">
+        <f>SUMIFS(Checklist!$H$2:$H$61,Checklist!$I$2:$I$61,"&lt;&gt;Done")</f>
+        <v>45.399999999999991</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" s="6" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="9" t="s">
         <v>0</v>
       </c>
@@ -3467,131 +3358,131 @@
         <v>151</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$A$2:$A$61,A7,Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B7" s="10">
+        <f>COUNTIFS(Checklist!$A$2:$A$61,A7,Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C7" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$A$2:$A$61,A7)</f>
+      <c r="C7" s="10">
+        <f>COUNTIF(Checklist!$A$2:$A$61,A7)</f>
         <v>3</v>
       </c>
-      <c r="D7" s="11" t="n">
-        <f aca="false">IF(C7=0,0,B7/C7)</f>
+      <c r="D7" s="11">
+        <f t="shared" ref="D7:D13" si="0">IF(C7=0,0,B7/C7)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$A$2:$A$61,A8,Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B8" s="10">
+        <f>COUNTIFS(Checklist!$A$2:$A$61,A8,Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C8" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$A$2:$A$61,A8)</f>
+      <c r="C8" s="10">
+        <f>COUNTIF(Checklist!$A$2:$A$61,A8)</f>
         <v>9</v>
       </c>
-      <c r="D8" s="11" t="n">
-        <f aca="false">IF(C8=0,0,B8/C8)</f>
+      <c r="D8" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$A$2:$A$61,A9,Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B9" s="10">
+        <f>COUNTIFS(Checklist!$A$2:$A$61,A9,Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C9" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$A$2:$A$61,A9)</f>
+      <c r="C9" s="10">
+        <f>COUNTIF(Checklist!$A$2:$A$61,A9)</f>
         <v>8</v>
       </c>
-      <c r="D9" s="11" t="n">
-        <f aca="false">IF(C9=0,0,B9/C9)</f>
+      <c r="D9" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B10" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$A$2:$A$61,A10,Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B10" s="10">
+        <f>COUNTIFS(Checklist!$A$2:$A$61,A10,Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C10" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$A$2:$A$61,A10)</f>
-        <v>17</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <f aca="false">IF(C10=0,0,B10/C10)</f>
+      <c r="C10" s="10">
+        <f>COUNTIF(Checklist!$A$2:$A$61,A10)</f>
+        <v>17</v>
+      </c>
+      <c r="D10" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B11" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$A$2:$A$61,A11,Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B11" s="10">
+        <f>COUNTIFS(Checklist!$A$2:$A$61,A11,Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C11" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$A$2:$A$61,A11)</f>
+      <c r="C11" s="10">
+        <f>COUNTIF(Checklist!$A$2:$A$61,A11)</f>
         <v>9</v>
       </c>
-      <c r="D11" s="11" t="n">
-        <f aca="false">IF(C11=0,0,B11/C11)</f>
+      <c r="D11" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="B12" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$A$2:$A$61,A12,Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B12" s="10">
+        <f>COUNTIFS(Checklist!$A$2:$A$61,A12,Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C12" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$A$2:$A$61,A12)</f>
+      <c r="C12" s="10">
+        <f>COUNTIF(Checklist!$A$2:$A$61,A12)</f>
         <v>8</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <f aca="false">IF(C12=0,0,B12/C12)</f>
+      <c r="D12" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$A$2:$A$61,A13,Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B13" s="10">
+        <f>COUNTIFS(Checklist!$A$2:$A$61,A13,Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C13" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$A$2:$A$61,A13)</f>
+      <c r="C13" s="10">
+        <f>COUNTIF(Checklist!$A$2:$A$61,A13)</f>
         <v>6</v>
       </c>
-      <c r="D13" s="11" t="n">
-        <f aca="false">IF(C13=0,0,B13/C13)</f>
+      <c r="D13" s="11">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="6" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="9" t="s">
         <v>3</v>
       </c>
@@ -3608,196 +3499,188 @@
         <v>153</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="B18" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$D$2:$D$61,"D1",Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B18" s="10">
+        <f>COUNTIFS(Checklist!$D$2:$D$61,"D1",Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C18" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$D$2:$D$61,"D1")</f>
+      <c r="C18" s="10">
+        <f>COUNTIF(Checklist!$D$2:$D$61,"D1")</f>
         <v>9</v>
       </c>
-      <c r="D18" s="11" t="n">
-        <f aca="false">IF(C18=0,0,B18/C18)</f>
+      <c r="D18" s="11">
+        <f t="shared" ref="D18:D23" si="1">IF(C18=0,0,B18/C18)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="11">
         <v>0.27</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="B19" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$D$2:$D$61,"D2",Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B19" s="10">
+        <f>COUNTIFS(Checklist!$D$2:$D$61,"D2",Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C19" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$D$2:$D$61,"D2")</f>
+      <c r="C19" s="10">
+        <f>COUNTIF(Checklist!$D$2:$D$61,"D2")</f>
         <v>8</v>
       </c>
-      <c r="D19" s="11" t="n">
-        <f aca="false">IF(C19=0,0,B19/C19)</f>
+      <c r="D19" s="11">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="11">
         <v>0.18</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="B20" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$D$2:$D$61,"D3",Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B20" s="10">
+        <f>COUNTIFS(Checklist!$D$2:$D$61,"D3",Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C20" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$D$2:$D$61,"D3")</f>
-        <v>17</v>
-      </c>
-      <c r="D20" s="11" t="n">
-        <f aca="false">IF(C20=0,0,B20/C20)</f>
+      <c r="C20" s="10">
+        <f>COUNTIF(Checklist!$D$2:$D$61,"D3")</f>
+        <v>17</v>
+      </c>
+      <c r="D20" s="11">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="11">
         <v>0.2</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="B21" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$D$2:$D$61,"D4",Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B21" s="10">
+        <f>COUNTIFS(Checklist!$D$2:$D$61,"D4",Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C21" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$D$2:$D$61,"D4")</f>
+      <c r="C21" s="10">
+        <f>COUNTIF(Checklist!$D$2:$D$61,"D4")</f>
         <v>9</v>
       </c>
-      <c r="D21" s="11" t="n">
-        <f aca="false">IF(C21=0,0,B21/C21)</f>
+      <c r="D21" s="11">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="11">
         <v>0.2</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="B22" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$D$2:$D$61,"D5",Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B22" s="10">
+        <f>COUNTIFS(Checklist!$D$2:$D$61,"D5",Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C22" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$D$2:$D$61,"D5")</f>
+      <c r="C22" s="10">
+        <f>COUNTIF(Checklist!$D$2:$D$61,"D5")</f>
         <v>8</v>
       </c>
-      <c r="D22" s="11" t="n">
-        <f aca="false">IF(C22=0,0,B22/C22)</f>
+      <c r="D22" s="11">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="11">
         <v>0.15</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="B23" s="10" t="n">
-        <f aca="false">COUNTIFS(Checklist!$D$2:$D$61,"ALL",Checklist!$I$2:$I$61,"Done")</f>
+      <c r="B23" s="10">
+        <f>COUNTIFS(Checklist!$D$2:$D$61,"ALL",Checklist!$I$2:$I$61,"Done")</f>
         <v>0</v>
       </c>
-      <c r="C23" s="10" t="n">
-        <f aca="false">COUNTIF(Checklist!$D$2:$D$61,"ALL")</f>
+      <c r="C23" s="10">
+        <f>COUNTIF(Checklist!$D$2:$D$61,"ALL")</f>
         <v>9</v>
       </c>
-      <c r="D23" s="11" t="n">
-        <f aca="false">IF(C23=0,0,B23/C23)</f>
+      <c r="D23" s="11">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E23" s="12"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" s="6" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" s="13" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" s="13" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" s="13" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" s="13" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" s="13" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" s="13" t="s">
         <v>166</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E41"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="65.19921875" customWidth="1"/>
+    <col min="4" max="4" width="42" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:5" ht="17.649999999999999" x14ac:dyDescent="0.5">
       <c r="A1" s="5" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="13" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="14" t="s">
         <v>1</v>
       </c>
@@ -3814,8 +3697,8 @@
         <v>171</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+    <row r="5" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A5" s="3">
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -3831,8 +3714,8 @@
         <v>174</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+    <row r="6" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A6" s="3">
         <v>2</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -3848,8 +3731,8 @@
         <v>177</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
+    <row r="7" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A7" s="3">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -3865,8 +3748,8 @@
         <v>180</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+    <row r="8" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A8" s="3">
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -3882,8 +3765,8 @@
         <v>183</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
+    <row r="9" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A9" s="3">
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -3899,8 +3782,8 @@
         <v>186</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+    <row r="10" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A10" s="3">
         <v>6</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -3916,8 +3799,8 @@
         <v>189</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
+    <row r="11" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A11" s="3">
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -3933,8 +3816,8 @@
         <v>192</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
+    <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A12" s="3">
         <v>8</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -3950,8 +3833,8 @@
         <v>195</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="n">
+    <row r="13" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A13" s="3">
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -3967,8 +3850,8 @@
         <v>198</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="n">
+    <row r="14" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A14" s="3">
         <v>10</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -3984,8 +3867,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="n">
+    <row r="15" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A15" s="3">
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -4001,8 +3884,8 @@
         <v>203</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="n">
+    <row r="16" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A16" s="3">
         <v>12</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -4018,8 +3901,8 @@
         <v>206</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="n">
+    <row r="17" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A17" s="3">
         <v>13</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -4035,8 +3918,8 @@
         <v>209</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="n">
+    <row r="18" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A18" s="3">
         <v>14</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -4052,8 +3935,8 @@
         <v>212</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="n">
+    <row r="19" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A19" s="3">
         <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -4069,8 +3952,8 @@
         <v>215</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="n">
+    <row r="20" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A20" s="3">
         <v>16</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -4086,8 +3969,8 @@
         <v>218</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="n">
+    <row r="21" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A21" s="3">
         <v>17</v>
       </c>
       <c r="B21" s="3" t="s">
@@ -4103,8 +3986,8 @@
         <v>221</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="n">
+    <row r="22" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A22" s="3">
         <v>18</v>
       </c>
       <c r="B22" s="3" t="s">
@@ -4120,8 +4003,8 @@
         <v>224</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="n">
+    <row r="23" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A23" s="3">
         <v>19</v>
       </c>
       <c r="B23" s="3" t="s">
@@ -4137,8 +4020,8 @@
         <v>227</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="n">
+    <row r="24" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A24" s="3">
         <v>20</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -4154,8 +4037,8 @@
         <v>230</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="n">
+    <row r="25" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A25" s="3">
         <v>21</v>
       </c>
       <c r="B25" s="3" t="s">
@@ -4171,8 +4054,8 @@
         <v>233</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="n">
+    <row r="26" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A26" s="3">
         <v>22</v>
       </c>
       <c r="B26" s="3" t="s">
@@ -4188,8 +4071,8 @@
         <v>236</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="n">
+    <row r="27" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+      <c r="A27" s="3">
         <v>23</v>
       </c>
       <c r="B27" s="3" t="s">
@@ -4205,8 +4088,8 @@
         <v>239</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="n">
+    <row r="28" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+      <c r="A28" s="3">
         <v>24</v>
       </c>
       <c r="B28" s="3" t="s">
@@ -4222,8 +4105,8 @@
         <v>206</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="n">
+    <row r="29" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A29" s="3">
         <v>25</v>
       </c>
       <c r="B29" s="3" t="s">
@@ -4239,8 +4122,8 @@
         <v>244</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="n">
+    <row r="30" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A30" s="3">
         <v>26</v>
       </c>
       <c r="B30" s="3" t="s">
@@ -4256,8 +4139,8 @@
         <v>244</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="n">
+    <row r="31" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A31" s="3">
         <v>27</v>
       </c>
       <c r="B31" s="3" t="s">
@@ -4273,8 +4156,8 @@
         <v>174</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="n">
+    <row r="32" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A32" s="3">
         <v>28</v>
       </c>
       <c r="B32" s="3" t="s">
@@ -4290,8 +4173,8 @@
         <v>244</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="n">
+    <row r="33" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+      <c r="A33" s="3">
         <v>29</v>
       </c>
       <c r="B33" s="3" t="s">
@@ -4307,8 +4190,8 @@
         <v>253</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="n">
+    <row r="34" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A34" s="3">
         <v>30</v>
       </c>
       <c r="B34" s="3" t="s">
@@ -4324,8 +4207,8 @@
         <v>256</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="n">
+    <row r="35" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A35" s="3">
         <v>31</v>
       </c>
       <c r="B35" s="3" t="s">
@@ -4341,8 +4224,8 @@
         <v>206</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="n">
+    <row r="36" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A36" s="3">
         <v>32</v>
       </c>
       <c r="B36" s="3" t="s">
@@ -4358,8 +4241,8 @@
         <v>260</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="n">
+    <row r="37" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A37" s="3">
         <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
@@ -4375,8 +4258,8 @@
         <v>263</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="n">
+    <row r="38" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A38" s="3">
         <v>34</v>
       </c>
       <c r="B38" s="3" t="s">
@@ -4392,8 +4275,8 @@
         <v>266</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="n">
+    <row r="39" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A39" s="3">
         <v>35</v>
       </c>
       <c r="B39" s="3" t="s">
@@ -4409,8 +4292,8 @@
         <v>269</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="n">
+    <row r="40" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+      <c r="A40" s="3">
         <v>36</v>
       </c>
       <c r="B40" s="3" t="s">
@@ -4426,8 +4309,8 @@
         <v>272</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="n">
+    <row r="41" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A41" s="3">
         <v>37</v>
       </c>
       <c r="B41" s="3" t="s">
@@ -4444,53 +4327,47 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E41"/>
+  <autoFilter ref="A4:E41" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <hyperlinks>
-    <hyperlink ref="E5" r:id="rId1" display="Tool use overview"/>
-    <hyperlink ref="E6" r:id="rId2" display="Sessions"/>
-    <hyperlink ref="E7" r:id="rId3" display="How we built our multi-agent research system"/>
-    <hyperlink ref="E8" r:id="rId4" display="Multi-agent research post ('Teach the orchestrator how to delegate')"/>
-    <hyperlink ref="E9" r:id="rId5" display="Subagents in Claude Code"/>
-    <hyperlink ref="E10" r:id="rId6" display="Subagents in the Agent SDK"/>
-    <hyperlink ref="E11" r:id="rId7" display="Building effective agents (orchestrator-workers)"/>
-    <hyperlink ref="E12" r:id="rId8" display="Permission modes (incl. plan mode)"/>
-    <hyperlink ref="E13" r:id="rId9" display="Multi-agent research post (checkpoints, resume-on-error)"/>
-    <hyperlink ref="E14" r:id="rId10" display="Building effective agents (the five workflow patterns)"/>
-    <hyperlink ref="E15" r:id="rId11" display="CLI reference + Headless"/>
-    <hyperlink ref="E16" r:id="rId12" display="Prompting best practices"/>
-    <hyperlink ref="E17" r:id="rId13" display="Code review"/>
-    <hyperlink ref="E18" r:id="rId14" display="Skills ('Run skills in a subagent')"/>
-    <hyperlink ref="E19" r:id="rId15" display="Common workflows (testing)"/>
-    <hyperlink ref="E20" r:id="rId16" display="Extend Claude Code"/>
-    <hyperlink ref="E21" r:id="rId17" display="Common workflows + Tools reference"/>
-    <hyperlink ref="E22" r:id="rId18" display="Multi-agent research post (appendix: subagent outputs)"/>
-    <hyperlink ref="E23" r:id="rId19" display="Multi-agent research post"/>
-    <hyperlink ref="E24" r:id="rId20" display="Effective context engineering for AI agents"/>
-    <hyperlink ref="E25" r:id="rId21" display="Context editing"/>
-    <hyperlink ref="E26" r:id="rId22" display="Exam-day one-pager"/>
-    <hyperlink ref="E27" r:id="rId23" display="Batch processing"/>
-    <hyperlink ref="E28" r:id="rId24" display="Prompting best practices"/>
-    <hyperlink ref="E29" r:id="rId25" display="Structured outputs"/>
-    <hyperlink ref="E30" r:id="rId26" display="Structured outputs"/>
-    <hyperlink ref="E31" r:id="rId27" display="Tool use overview"/>
-    <hyperlink ref="E32" r:id="rId28" display="Structured outputs"/>
-    <hyperlink ref="E33" r:id="rId29" display="Structured outputs + Prompting best practices"/>
-    <hyperlink ref="E34" r:id="rId30" display="Memory + Code review"/>
-    <hyperlink ref="E35" r:id="rId31" display="Prompting best practices"/>
-    <hyperlink ref="E36" r:id="rId32" display="Tools reference"/>
-    <hyperlink ref="E37" r:id="rId33" display="Subagents + Tool use overview"/>
-    <hyperlink ref="E38" r:id="rId34" display="Model Context Protocol docs"/>
-    <hyperlink ref="E39" r:id="rId35" display="MCP in Claude Code"/>
-    <hyperlink ref="E40" r:id="rId36" display="Tool use overview + MCP docs"/>
-    <hyperlink ref="E41" r:id="rId37" display="Tool use overview"/>
+    <hyperlink ref="E5" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="E7" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
+    <hyperlink ref="E8" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
+    <hyperlink ref="E9" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="E10" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="E11" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="E12" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
+    <hyperlink ref="E13" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
+    <hyperlink ref="E14" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="E15" r:id="rId11" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
+    <hyperlink ref="E16" r:id="rId12" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
+    <hyperlink ref="E17" r:id="rId13" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
+    <hyperlink ref="E18" r:id="rId14" xr:uid="{00000000-0004-0000-0200-00000D000000}"/>
+    <hyperlink ref="E19" r:id="rId15" xr:uid="{00000000-0004-0000-0200-00000E000000}"/>
+    <hyperlink ref="E20" r:id="rId16" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
+    <hyperlink ref="E21" r:id="rId17" xr:uid="{00000000-0004-0000-0200-000010000000}"/>
+    <hyperlink ref="E22" r:id="rId18" xr:uid="{00000000-0004-0000-0200-000011000000}"/>
+    <hyperlink ref="E23" r:id="rId19" xr:uid="{00000000-0004-0000-0200-000012000000}"/>
+    <hyperlink ref="E24" r:id="rId20" xr:uid="{00000000-0004-0000-0200-000013000000}"/>
+    <hyperlink ref="E25" r:id="rId21" xr:uid="{00000000-0004-0000-0200-000014000000}"/>
+    <hyperlink ref="E26" r:id="rId22" xr:uid="{00000000-0004-0000-0200-000015000000}"/>
+    <hyperlink ref="E27" r:id="rId23" xr:uid="{00000000-0004-0000-0200-000016000000}"/>
+    <hyperlink ref="E28" r:id="rId24" xr:uid="{00000000-0004-0000-0200-000017000000}"/>
+    <hyperlink ref="E29" r:id="rId25" xr:uid="{00000000-0004-0000-0200-000018000000}"/>
+    <hyperlink ref="E30" r:id="rId26" xr:uid="{00000000-0004-0000-0200-000019000000}"/>
+    <hyperlink ref="E31" r:id="rId27" xr:uid="{00000000-0004-0000-0200-00001A000000}"/>
+    <hyperlink ref="E32" r:id="rId28" xr:uid="{00000000-0004-0000-0200-00001B000000}"/>
+    <hyperlink ref="E33" r:id="rId29" xr:uid="{00000000-0004-0000-0200-00001C000000}"/>
+    <hyperlink ref="E34" r:id="rId30" xr:uid="{00000000-0004-0000-0200-00001D000000}"/>
+    <hyperlink ref="E35" r:id="rId31" xr:uid="{00000000-0004-0000-0200-00001E000000}"/>
+    <hyperlink ref="E36" r:id="rId32" xr:uid="{00000000-0004-0000-0200-00001F000000}"/>
+    <hyperlink ref="E37" r:id="rId33" xr:uid="{00000000-0004-0000-0200-000020000000}"/>
+    <hyperlink ref="E38" r:id="rId34" xr:uid="{00000000-0004-0000-0200-000021000000}"/>
+    <hyperlink ref="E39" r:id="rId35" xr:uid="{00000000-0004-0000-0200-000022000000}"/>
+    <hyperlink ref="E40" r:id="rId36" xr:uid="{00000000-0004-0000-0200-000023000000}"/>
+    <hyperlink ref="E41" r:id="rId37" xr:uid="{00000000-0004-0000-0200-000024000000}"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId38"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add D1L12 lab on agent design judgment and update gitignore with event/facilitation directories
</commit_message>
<xml_diff>
--- a/CCAF-Study-Checklist.xlsx
+++ b/CCAF-Study-Checklist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\Russel-QL2\_Dev\Claude-Learning-Exercises\CCAF-StudyGuide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DEDC5DE-1A39-4B71-ACD4-6018B70C8340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A203A5-4E3C-4A0D-8A68-DF85450DD9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist" sheetId="1" r:id="rId1"/>
@@ -876,7 +876,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -914,6 +914,17 @@
       <sz val="10"/>
       <name val="Arial"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -957,7 +968,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -982,6 +993,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3665,7 +3682,7 @@
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="65.19921875" customWidth="1"/>
+    <col min="3" max="3" width="75.73046875" customWidth="1"/>
     <col min="4" max="4" width="42" customWidth="1"/>
     <col min="5" max="5" width="34" customWidth="1"/>
   </cols>
@@ -3697,7 +3714,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>1</v>
       </c>
@@ -3714,7 +3731,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A6" s="3">
         <v>2</v>
       </c>
@@ -3731,14 +3748,14 @@
         <v>177</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" ht="39.4" x14ac:dyDescent="0.45">
       <c r="A7" s="3">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="15" t="s">
         <v>178</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -3748,7 +3765,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A8" s="3">
         <v>4</v>
       </c>
@@ -3782,7 +3799,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A10" s="3">
         <v>6</v>
       </c>
@@ -3799,7 +3816,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A11" s="3">
         <v>7</v>
       </c>
@@ -3816,358 +3833,358 @@
         <v>192</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A12" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A13" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A14" s="3">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>191</v>
+        <v>223</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A15" s="3">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>201</v>
+        <v>225</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A16" s="3">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>105</v>
+        <v>51</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>204</v>
+        <v>261</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>205</v>
+        <v>262</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A17" s="3">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>207</v>
+        <v>264</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>208</v>
+        <v>265</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A18" s="3">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>210</v>
+        <v>267</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>211</v>
+        <v>268</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A19" s="3">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>213</v>
+        <v>270</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>214</v>
+        <v>271</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="39.4" x14ac:dyDescent="0.45">
       <c r="A20" s="3">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>216</v>
+        <v>51</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>273</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>217</v>
+        <v>274</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A21" s="3">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>66</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>219</v>
+        <v>193</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>220</v>
+        <v>194</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A22" s="3">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>223</v>
+        <v>202</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A23" s="3">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>225</v>
+        <v>207</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A24" s="3">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>120</v>
+        <v>66</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A25" s="3">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>120</v>
+        <v>66</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>231</v>
+        <v>213</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="52.5" x14ac:dyDescent="0.45">
       <c r="A26" s="3">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>234</v>
+        <v>66</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>216</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>236</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A27" s="3">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>120</v>
+        <v>66</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>237</v>
+        <v>219</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A28" s="3">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>105</v>
+        <v>66</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A29" s="3">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>105</v>
+        <v>66</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>242</v>
+        <v>259</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>243</v>
+        <v>220</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A30" s="3">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>105</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>246</v>
+        <v>205</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="51" x14ac:dyDescent="0.45">
       <c r="A31" s="3">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>105</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A32" s="3">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>249</v>
+      <c r="C32" s="16" t="s">
+        <v>242</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>244</v>
@@ -4175,159 +4192,163 @@
     </row>
     <row r="33" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A33" s="3">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>105</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="52.5" x14ac:dyDescent="0.45">
       <c r="A34" s="3">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>254</v>
+        <v>105</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>247</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A35" s="3">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>105</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+      <c r="A36" s="3">
+        <v>29</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+      <c r="A37" s="3">
+        <v>31</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E37" s="4" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
-      <c r="A36" s="3">
-        <v>32</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
-      <c r="A37" s="3">
-        <v>33</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A38" s="3">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>264</v>
+        <v>228</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>265</v>
+        <v>229</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A39" s="3">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>267</v>
+        <v>231</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>268</v>
+        <v>232</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>269</v>
+        <v>233</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A40" s="3">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>270</v>
+        <v>234</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>271</v>
+        <v>235</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="52.5" x14ac:dyDescent="0.45">
       <c r="A41" s="3">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>273</v>
+        <v>120</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>237</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>274</v>
+        <v>238</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>174</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E41" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A4:E41" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:E41">
+      <sortCondition ref="B4:B41"/>
+    </sortState>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="E5" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
     <hyperlink ref="E6" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
@@ -4336,36 +4357,36 @@
     <hyperlink ref="E9" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
     <hyperlink ref="E10" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
     <hyperlink ref="E11" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
-    <hyperlink ref="E12" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
-    <hyperlink ref="E13" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
-    <hyperlink ref="E14" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
-    <hyperlink ref="E15" r:id="rId11" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
-    <hyperlink ref="E16" r:id="rId12" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
-    <hyperlink ref="E17" r:id="rId13" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
-    <hyperlink ref="E18" r:id="rId14" xr:uid="{00000000-0004-0000-0200-00000D000000}"/>
-    <hyperlink ref="E19" r:id="rId15" xr:uid="{00000000-0004-0000-0200-00000E000000}"/>
-    <hyperlink ref="E20" r:id="rId16" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
-    <hyperlink ref="E21" r:id="rId17" xr:uid="{00000000-0004-0000-0200-000010000000}"/>
-    <hyperlink ref="E22" r:id="rId18" xr:uid="{00000000-0004-0000-0200-000011000000}"/>
-    <hyperlink ref="E23" r:id="rId19" xr:uid="{00000000-0004-0000-0200-000012000000}"/>
-    <hyperlink ref="E24" r:id="rId20" xr:uid="{00000000-0004-0000-0200-000013000000}"/>
-    <hyperlink ref="E25" r:id="rId21" xr:uid="{00000000-0004-0000-0200-000014000000}"/>
-    <hyperlink ref="E26" r:id="rId22" xr:uid="{00000000-0004-0000-0200-000015000000}"/>
-    <hyperlink ref="E27" r:id="rId23" xr:uid="{00000000-0004-0000-0200-000016000000}"/>
-    <hyperlink ref="E28" r:id="rId24" xr:uid="{00000000-0004-0000-0200-000017000000}"/>
-    <hyperlink ref="E29" r:id="rId25" xr:uid="{00000000-0004-0000-0200-000018000000}"/>
-    <hyperlink ref="E30" r:id="rId26" xr:uid="{00000000-0004-0000-0200-000019000000}"/>
-    <hyperlink ref="E31" r:id="rId27" xr:uid="{00000000-0004-0000-0200-00001A000000}"/>
-    <hyperlink ref="E32" r:id="rId28" xr:uid="{00000000-0004-0000-0200-00001B000000}"/>
-    <hyperlink ref="E33" r:id="rId29" xr:uid="{00000000-0004-0000-0200-00001C000000}"/>
-    <hyperlink ref="E34" r:id="rId30" xr:uid="{00000000-0004-0000-0200-00001D000000}"/>
-    <hyperlink ref="E35" r:id="rId31" xr:uid="{00000000-0004-0000-0200-00001E000000}"/>
-    <hyperlink ref="E36" r:id="rId32" xr:uid="{00000000-0004-0000-0200-00001F000000}"/>
-    <hyperlink ref="E37" r:id="rId33" xr:uid="{00000000-0004-0000-0200-000020000000}"/>
-    <hyperlink ref="E38" r:id="rId34" xr:uid="{00000000-0004-0000-0200-000021000000}"/>
-    <hyperlink ref="E39" r:id="rId35" xr:uid="{00000000-0004-0000-0200-000022000000}"/>
-    <hyperlink ref="E40" r:id="rId36" xr:uid="{00000000-0004-0000-0200-000023000000}"/>
-    <hyperlink ref="E41" r:id="rId37" xr:uid="{00000000-0004-0000-0200-000024000000}"/>
+    <hyperlink ref="E21" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
+    <hyperlink ref="E12" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
+    <hyperlink ref="E13" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="E22" r:id="rId11" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
+    <hyperlink ref="E30" r:id="rId12" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
+    <hyperlink ref="E23" r:id="rId13" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
+    <hyperlink ref="E24" r:id="rId14" xr:uid="{00000000-0004-0000-0200-00000D000000}"/>
+    <hyperlink ref="E25" r:id="rId15" xr:uid="{00000000-0004-0000-0200-00000E000000}"/>
+    <hyperlink ref="E26" r:id="rId16" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
+    <hyperlink ref="E27" r:id="rId17" xr:uid="{00000000-0004-0000-0200-000010000000}"/>
+    <hyperlink ref="E14" r:id="rId18" xr:uid="{00000000-0004-0000-0200-000011000000}"/>
+    <hyperlink ref="E15" r:id="rId19" xr:uid="{00000000-0004-0000-0200-000012000000}"/>
+    <hyperlink ref="E38" r:id="rId20" xr:uid="{00000000-0004-0000-0200-000013000000}"/>
+    <hyperlink ref="E39" r:id="rId21" xr:uid="{00000000-0004-0000-0200-000014000000}"/>
+    <hyperlink ref="E40" r:id="rId22" xr:uid="{00000000-0004-0000-0200-000015000000}"/>
+    <hyperlink ref="E41" r:id="rId23" xr:uid="{00000000-0004-0000-0200-000016000000}"/>
+    <hyperlink ref="E31" r:id="rId24" xr:uid="{00000000-0004-0000-0200-000017000000}"/>
+    <hyperlink ref="E32" r:id="rId25" xr:uid="{00000000-0004-0000-0200-000018000000}"/>
+    <hyperlink ref="E33" r:id="rId26" xr:uid="{00000000-0004-0000-0200-000019000000}"/>
+    <hyperlink ref="E34" r:id="rId27" xr:uid="{00000000-0004-0000-0200-00001A000000}"/>
+    <hyperlink ref="E35" r:id="rId28" xr:uid="{00000000-0004-0000-0200-00001B000000}"/>
+    <hyperlink ref="E36" r:id="rId29" xr:uid="{00000000-0004-0000-0200-00001C000000}"/>
+    <hyperlink ref="E28" r:id="rId30" xr:uid="{00000000-0004-0000-0200-00001D000000}"/>
+    <hyperlink ref="E37" r:id="rId31" xr:uid="{00000000-0004-0000-0200-00001E000000}"/>
+    <hyperlink ref="E29" r:id="rId32" xr:uid="{00000000-0004-0000-0200-00001F000000}"/>
+    <hyperlink ref="E16" r:id="rId33" xr:uid="{00000000-0004-0000-0200-000020000000}"/>
+    <hyperlink ref="E17" r:id="rId34" xr:uid="{00000000-0004-0000-0200-000021000000}"/>
+    <hyperlink ref="E18" r:id="rId35" xr:uid="{00000000-0004-0000-0200-000022000000}"/>
+    <hyperlink ref="E19" r:id="rId36" xr:uid="{00000000-0004-0000-0200-000023000000}"/>
+    <hyperlink ref="E20" r:id="rId37" xr:uid="{00000000-0004-0000-0200-000024000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
feat: add multiple hands-on lab notebooks and update study checklist
</commit_message>
<xml_diff>
--- a/CCAF-Study-Checklist.xlsx
+++ b/CCAF-Study-Checklist.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A203A5-4E3C-4A0D-8A68-DF85450DD9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist" sheetId="1" r:id="rId1"/>
@@ -3714,7 +3714,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>1</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A6" s="3">
         <v>2</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A10" s="3">
         <v>6</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A12" s="3">
         <v>9</v>
       </c>
@@ -3867,7 +3867,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A14" s="3">
         <v>18</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A17" s="3">
         <v>34</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A21" s="3">
         <v>8</v>
       </c>
@@ -4071,7 +4071,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" ht="39.4" x14ac:dyDescent="0.45">
       <c r="A26" s="3">
         <v>16</v>
       </c>
@@ -4088,7 +4088,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A27" s="3">
         <v>17</v>
       </c>
@@ -4105,7 +4105,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A28" s="3">
         <v>30</v>
       </c>
@@ -4122,7 +4122,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A29" s="3">
         <v>32</v>
       </c>
@@ -4156,7 +4156,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="51" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A31" s="3">
         <v>24</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:5" ht="39.4" x14ac:dyDescent="0.45">
       <c r="A34" s="3">
         <v>27</v>
       </c>
@@ -4258,7 +4258,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:5" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A37" s="3">
         <v>31</v>
       </c>
@@ -4326,7 +4326,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:5" ht="39.4" x14ac:dyDescent="0.45">
       <c r="A41" s="3">
         <v>23</v>
       </c>

</xml_diff>